<commit_message>
Bug fixes and e4 split map work!
</commit_message>
<xml_diff>
--- a/stuff/pokemon game.xlsx
+++ b/stuff/pokemon game.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A40537B-5722-42CA-A098-78563B4DB0E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC8B703-1874-4CD0-B367-3F3D92BB25B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7BD02A17-B686-4FC4-8065-C777F779E0C9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3209" uniqueCount="1672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3210" uniqueCount="1673">
   <si>
     <t>Leafer</t>
   </si>
@@ -5052,6 +5052,9 @@
   </si>
   <si>
     <t>Icy Serpent: Dragon Dance/Sword of Dawn/Ice Spinner/Earthquake/Magic Fang/Magic Reflect</t>
+  </si>
+  <si>
+    <t>Move Encyclopedia</t>
   </si>
 </sst>
 </file>
@@ -5775,10 +5778,10 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CCCD70F4-8B57-40C5-9200-528EDFFF7692}" name="Table5" displayName="Table5" ref="AK29:AN426" totalsRowShown="0">
-  <autoFilter ref="AK29:AN426" xr:uid="{CCCD70F4-8B57-40C5-9200-528EDFFF7692}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="AK30:AN426">
-    <sortCondition ref="AM29:AM426"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CCCD70F4-8B57-40C5-9200-528EDFFF7692}" name="Table5" displayName="Table5" ref="AK29:AN427" totalsRowShown="0">
+  <autoFilter ref="AK29:AN427" xr:uid="{CCCD70F4-8B57-40C5-9200-528EDFFF7692}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="AK30:AN427">
+    <sortCondition ref="AM29:AM427"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{26A53F18-86E2-4791-9F01-3774B056CCDA}" name="Pos"/>
@@ -15549,7 +15552,7 @@
         <v>301</v>
       </c>
       <c r="AL122" t="s">
-        <v>1381</v>
+        <v>1672</v>
       </c>
       <c r="AM122">
         <v>0</v>
@@ -15619,10 +15622,10 @@
         <v>1.4E-3</v>
       </c>
       <c r="AK123">
-        <v>333</v>
+        <v>302</v>
       </c>
       <c r="AL123" t="s">
-        <v>1351</v>
+        <v>1381</v>
       </c>
       <c r="AM123">
         <v>0</v>
@@ -15692,16 +15695,13 @@
         <v>1.4E-3</v>
       </c>
       <c r="AK124">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="AL124" t="s">
-        <v>1266</v>
+        <v>1351</v>
       </c>
       <c r="AM124">
         <v>0</v>
-      </c>
-      <c r="AN124" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="125" spans="2:40" x14ac:dyDescent="0.25">
@@ -15768,13 +15768,16 @@
         <v>1.4E-3</v>
       </c>
       <c r="AK125">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="AL125" t="s">
-        <v>1415</v>
+        <v>1266</v>
       </c>
       <c r="AM125">
         <v>0</v>
+      </c>
+      <c r="AN125" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="126" spans="2:40" x14ac:dyDescent="0.25">
@@ -15844,7 +15847,7 @@
         <v>355</v>
       </c>
       <c r="AL126" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="AM126">
         <v>0</v>
@@ -15917,7 +15920,7 @@
         <v>356</v>
       </c>
       <c r="AL127" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="AM127">
         <v>0</v>
@@ -15990,7 +15993,7 @@
         <v>357</v>
       </c>
       <c r="AL128" t="s">
-        <v>1418</v>
+        <v>1417</v>
       </c>
       <c r="AM128">
         <v>0</v>
@@ -16063,7 +16066,7 @@
         <v>358</v>
       </c>
       <c r="AL129" t="s">
-        <v>1472</v>
+        <v>1418</v>
       </c>
       <c r="AM129">
         <v>0</v>
@@ -16136,7 +16139,7 @@
         <v>359</v>
       </c>
       <c r="AL130" t="s">
-        <v>1388</v>
+        <v>1472</v>
       </c>
       <c r="AM130">
         <v>0</v>
@@ -16209,7 +16212,7 @@
         <v>360</v>
       </c>
       <c r="AL131" t="s">
-        <v>1474</v>
+        <v>1388</v>
       </c>
       <c r="AM131">
         <v>0</v>
@@ -16282,7 +16285,7 @@
         <v>361</v>
       </c>
       <c r="AL132" t="s">
-        <v>1471</v>
+        <v>1474</v>
       </c>
       <c r="AM132">
         <v>0</v>
@@ -16355,7 +16358,7 @@
         <v>362</v>
       </c>
       <c r="AL133" t="s">
-        <v>1403</v>
+        <v>1471</v>
       </c>
       <c r="AM133">
         <v>0</v>
@@ -16428,7 +16431,7 @@
         <v>363</v>
       </c>
       <c r="AL134" t="s">
-        <v>1394</v>
+        <v>1403</v>
       </c>
       <c r="AM134">
         <v>0</v>
@@ -16498,10 +16501,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK135">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="AL135" t="s">
-        <v>1408</v>
+        <v>1394</v>
       </c>
       <c r="AM135">
         <v>0</v>
@@ -16571,10 +16574,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK136">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="AL136" t="s">
-        <v>1387</v>
+        <v>1408</v>
       </c>
       <c r="AM136">
         <v>0</v>
@@ -16643,8 +16646,11 @@
       <c r="AI137" s="35">
         <v>2.0999999999999999E-3</v>
       </c>
+      <c r="AK137">
+        <v>369</v>
+      </c>
       <c r="AL137" t="s">
-        <v>1641</v>
+        <v>1387</v>
       </c>
       <c r="AM137">
         <v>0</v>
@@ -16717,7 +16723,7 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AL138" t="s">
-        <v>1642</v>
+        <v>1641</v>
       </c>
       <c r="AM138">
         <v>0</v>
@@ -16787,7 +16793,7 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AL139" t="s">
-        <v>1651</v>
+        <v>1642</v>
       </c>
       <c r="AM139">
         <v>0</v>
@@ -16857,7 +16863,7 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AL140" t="s">
-        <v>1662</v>
+        <v>1651</v>
       </c>
       <c r="AM140">
         <v>0</v>
@@ -16933,14 +16939,11 @@
       <c r="AI141" s="35">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="AK141">
-        <v>73</v>
-      </c>
       <c r="AL141" t="s">
-        <v>1271</v>
+        <v>1662</v>
       </c>
       <c r="AM141">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142" spans="2:39" x14ac:dyDescent="0.25">
@@ -17017,10 +17020,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK142">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="AL142" t="s">
-        <v>1228</v>
+        <v>1271</v>
       </c>
       <c r="AM142">
         <v>1</v>
@@ -17097,10 +17100,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK143">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AL143" t="s">
-        <v>1367</v>
+        <v>1228</v>
       </c>
       <c r="AM143">
         <v>1</v>
@@ -17189,10 +17192,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK144">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AL144" t="s">
-        <v>1281</v>
+        <v>1367</v>
       </c>
       <c r="AM144">
         <v>1</v>
@@ -17274,10 +17277,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK145">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AL145" t="s">
-        <v>1233</v>
+        <v>1281</v>
       </c>
       <c r="AM145">
         <v>1</v>
@@ -17384,10 +17387,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK146">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AL146" t="s">
-        <v>881</v>
+        <v>1233</v>
       </c>
       <c r="AM146">
         <v>1</v>
@@ -17491,10 +17494,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK147">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AL147" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="AM147">
         <v>1</v>
@@ -17598,10 +17601,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK148">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AL148" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="AM148">
         <v>1</v>
@@ -17705,10 +17708,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK149">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AL149" t="s">
-        <v>897</v>
+        <v>883</v>
       </c>
       <c r="AM149">
         <v>1</v>
@@ -17812,16 +17815,13 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK150">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AL150" t="s">
-        <v>879</v>
+        <v>897</v>
       </c>
       <c r="AM150">
         <v>1</v>
-      </c>
-      <c r="AN150" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="151" spans="1:40" x14ac:dyDescent="0.25">
@@ -17919,10 +17919,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK151">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AL151" t="s">
-        <v>891</v>
+        <v>879</v>
       </c>
       <c r="AM151">
         <v>1</v>
@@ -18032,13 +18032,16 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK152">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AL152" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="AM152">
         <v>1</v>
+      </c>
+      <c r="AN152" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="153" spans="1:40" x14ac:dyDescent="0.25">
@@ -18139,10 +18142,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK153">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="AL153" t="s">
-        <v>1640</v>
+        <v>890</v>
       </c>
       <c r="AM153">
         <v>1</v>
@@ -18243,10 +18246,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK154">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AL154" t="s">
-        <v>886</v>
+        <v>1640</v>
       </c>
       <c r="AM154">
         <v>1</v>
@@ -18350,10 +18353,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK155">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AL155" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="AM155">
         <v>1</v>
@@ -18457,10 +18460,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK156">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AL156" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="AM156">
         <v>1</v>
@@ -18564,10 +18567,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK157">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AL157" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="AM157">
         <v>1</v>
@@ -18671,10 +18674,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK158">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AL158" t="s">
-        <v>878</v>
+        <v>889</v>
       </c>
       <c r="AM158">
         <v>1</v>
@@ -18778,10 +18781,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK159">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AL159" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="AM159">
         <v>1</v>
@@ -18882,10 +18885,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK160">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AL160" t="s">
-        <v>892</v>
+        <v>880</v>
       </c>
       <c r="AM160">
         <v>1</v>
@@ -18989,16 +18992,13 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK161">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AL161" t="s">
-        <v>1476</v>
+        <v>892</v>
       </c>
       <c r="AM161">
         <v>1</v>
-      </c>
-      <c r="AN161" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="162" spans="1:40" x14ac:dyDescent="0.25">
@@ -19099,13 +19099,16 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK162">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AL162" t="s">
-        <v>988</v>
+        <v>1476</v>
       </c>
       <c r="AM162">
         <v>1</v>
+      </c>
+      <c r="AN162" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="163" spans="1:40" x14ac:dyDescent="0.25">
@@ -19206,10 +19209,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK163">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AL163" t="s">
-        <v>1477</v>
+        <v>988</v>
       </c>
       <c r="AM163">
         <v>1</v>
@@ -19316,10 +19319,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK164">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AL164" t="s">
-        <v>898</v>
+        <v>1477</v>
       </c>
       <c r="AM164">
         <v>1</v>
@@ -19423,10 +19426,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK165">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="AL165" t="s">
-        <v>906</v>
+        <v>898</v>
       </c>
       <c r="AM165">
         <v>1</v>
@@ -19527,16 +19530,13 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK166">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AL166" t="s">
-        <v>1643</v>
+        <v>906</v>
       </c>
       <c r="AM166">
         <v>1</v>
-      </c>
-      <c r="AN166" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="167" spans="1:40" x14ac:dyDescent="0.25">
@@ -19635,10 +19635,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK167">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AL167" t="s">
-        <v>904</v>
+        <v>1643</v>
       </c>
       <c r="AM167">
         <v>1</v>
@@ -19743,13 +19743,16 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK168">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AL168" t="s">
-        <v>1478</v>
+        <v>904</v>
       </c>
       <c r="AM168">
         <v>1</v>
+      </c>
+      <c r="AN168" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="169" spans="1:40" x14ac:dyDescent="0.25">
@@ -19847,10 +19850,10 @@
         <v>2.0999999999999999E-3</v>
       </c>
       <c r="AK169">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AL169" t="s">
-        <v>1479</v>
+        <v>1478</v>
       </c>
       <c r="AM169">
         <v>1</v>
@@ -19954,10 +19957,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK170">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AL170" t="s">
-        <v>899</v>
+        <v>1479</v>
       </c>
       <c r="AM170">
         <v>1</v>
@@ -20059,10 +20062,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK171">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="AL171" t="s">
-        <v>1014</v>
+        <v>899</v>
       </c>
       <c r="AM171">
         <v>1</v>
@@ -20164,10 +20167,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK172">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="AL172" t="s">
-        <v>903</v>
+        <v>1014</v>
       </c>
       <c r="AM172">
         <v>1</v>
@@ -20263,10 +20266,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK173">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AL173" t="s">
-        <v>909</v>
+        <v>903</v>
       </c>
       <c r="AM173">
         <v>1</v>
@@ -20367,10 +20370,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK174">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="AL174" t="s">
-        <v>1481</v>
+        <v>909</v>
       </c>
       <c r="AM174">
         <v>1</v>
@@ -20471,10 +20474,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK175">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="AL175" t="s">
-        <v>902</v>
+        <v>1481</v>
       </c>
       <c r="AM175">
         <v>1</v>
@@ -20572,10 +20575,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK176">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL176" t="s">
-        <v>1015</v>
+        <v>902</v>
       </c>
       <c r="AM176">
         <v>1</v>
@@ -20674,10 +20677,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK177">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AL177" t="s">
-        <v>884</v>
+        <v>1015</v>
       </c>
       <c r="AM177">
         <v>1</v>
@@ -20776,10 +20779,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK178">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="AL178" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="AM178">
         <v>1</v>
@@ -20875,10 +20878,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK179">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AL179" t="s">
-        <v>1366</v>
+        <v>885</v>
       </c>
       <c r="AM179">
         <v>1</v>
@@ -20977,10 +20980,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK180">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="AL180" t="s">
-        <v>895</v>
+        <v>1366</v>
       </c>
       <c r="AM180">
         <v>1</v>
@@ -21079,10 +21082,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK181">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AL181" t="s">
-        <v>1238</v>
+        <v>895</v>
       </c>
       <c r="AM181">
         <v>1</v>
@@ -21178,10 +21181,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK182">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AL182" t="s">
-        <v>1250</v>
+        <v>1238</v>
       </c>
       <c r="AM182">
         <v>1</v>
@@ -21279,16 +21282,13 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK183">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AL183" t="s">
-        <v>1060</v>
+        <v>1250</v>
       </c>
       <c r="AM183">
         <v>1</v>
-      </c>
-      <c r="AN183" t="s">
-        <v>1564</v>
       </c>
     </row>
     <row r="184" spans="1:40" x14ac:dyDescent="0.25">
@@ -21389,13 +21389,16 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK184">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="AL184" t="s">
-        <v>900</v>
+        <v>1060</v>
       </c>
       <c r="AM184">
         <v>1</v>
+      </c>
+      <c r="AN184" t="s">
+        <v>1564</v>
       </c>
     </row>
     <row r="185" spans="1:40" x14ac:dyDescent="0.25">
@@ -21493,10 +21496,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK185">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AL185" t="s">
-        <v>910</v>
+        <v>900</v>
       </c>
       <c r="AM185">
         <v>1</v>
@@ -21597,10 +21600,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK186">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="AL186" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="AM186">
         <v>1</v>
@@ -21701,10 +21704,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK187">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="AL187" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="AM187">
         <v>1</v>
@@ -21802,10 +21805,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK188">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="AL188" t="s">
-        <v>928</v>
+        <v>912</v>
       </c>
       <c r="AM188">
         <v>1</v>
@@ -21904,10 +21907,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK189">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AL189" t="s">
-        <v>914</v>
+        <v>928</v>
       </c>
       <c r="AM189">
         <v>1</v>
@@ -22006,16 +22009,13 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK190">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AL190" t="s">
-        <v>929</v>
+        <v>914</v>
       </c>
       <c r="AM190">
         <v>1</v>
-      </c>
-      <c r="AN190" t="s">
-        <v>1564</v>
       </c>
     </row>
     <row r="191" spans="1:40" x14ac:dyDescent="0.25">
@@ -22108,10 +22108,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK191">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AL191" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="AM191">
         <v>1</v>
@@ -22206,13 +22206,16 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK192">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AL192" t="s">
-        <v>915</v>
+        <v>930</v>
       </c>
       <c r="AM192">
         <v>1</v>
+      </c>
+      <c r="AN192" t="s">
+        <v>1564</v>
       </c>
     </row>
     <row r="193" spans="1:40" x14ac:dyDescent="0.25">
@@ -22304,10 +22307,10 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="AK193">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AL193" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="AM193">
         <v>1</v>
@@ -22408,10 +22411,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK194">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AL194" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="AM194">
         <v>1</v>
@@ -22509,10 +22512,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK195">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="AL195" t="s">
-        <v>920</v>
+        <v>917</v>
       </c>
       <c r="AM195">
         <v>1</v>
@@ -22613,10 +22616,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK196">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AL196" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="AM196">
         <v>1</v>
@@ -22717,10 +22720,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK197">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AL197" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="AM197">
         <v>1</v>
@@ -22821,16 +22824,13 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK198">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="AL198" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="AM198">
         <v>1</v>
-      </c>
-      <c r="AN198" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="199" spans="1:40" x14ac:dyDescent="0.25">
@@ -22925,13 +22925,16 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK199">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AL199" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="AM199">
         <v>1</v>
+      </c>
+      <c r="AN199" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="200" spans="1:40" x14ac:dyDescent="0.25">
@@ -23029,10 +23032,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK200">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AL200" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="AM200">
         <v>1</v>
@@ -23130,10 +23133,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK201">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AL201" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="AM201">
         <v>1</v>
@@ -23231,10 +23234,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK202">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AL202" t="s">
-        <v>1538</v>
+        <v>927</v>
       </c>
       <c r="AM202">
         <v>1</v>
@@ -23329,10 +23332,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK203">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="AL203" t="s">
-        <v>1348</v>
+        <v>1538</v>
       </c>
       <c r="AM203">
         <v>1</v>
@@ -23430,10 +23433,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK204">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="AL204" t="s">
-        <v>1353</v>
+        <v>1348</v>
       </c>
       <c r="AM204">
         <v>1</v>
@@ -23528,10 +23531,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK205">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AL205" t="s">
-        <v>1407</v>
+        <v>1353</v>
       </c>
       <c r="AM205">
         <v>1</v>
@@ -23626,10 +23629,10 @@
         <v>3.3999999999999998E-3</v>
       </c>
       <c r="AK206">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AL206" t="s">
-        <v>1483</v>
+        <v>1407</v>
       </c>
       <c r="AM206">
         <v>1</v>
@@ -23727,10 +23730,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK207">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AL207" t="s">
-        <v>1484</v>
+        <v>1483</v>
       </c>
       <c r="AM207">
         <v>1</v>
@@ -23822,10 +23825,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK208">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AL208" t="s">
-        <v>1485</v>
+        <v>1484</v>
       </c>
       <c r="AM208">
         <v>1</v>
@@ -23918,10 +23921,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK209">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AL209" t="s">
-        <v>1486</v>
+        <v>1485</v>
       </c>
       <c r="AM209">
         <v>1</v>
@@ -24011,10 +24014,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK210">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AL210" t="s">
-        <v>1487</v>
+        <v>1486</v>
       </c>
       <c r="AM210">
         <v>1</v>
@@ -24109,16 +24112,13 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK211">
-        <v>191</v>
+        <v>159</v>
       </c>
       <c r="AL211" t="s">
-        <v>1245</v>
+        <v>1487</v>
       </c>
       <c r="AM211">
         <v>1</v>
-      </c>
-      <c r="AN211" t="s">
-        <v>1565</v>
       </c>
     </row>
     <row r="212" spans="1:40" x14ac:dyDescent="0.25">
@@ -24207,13 +24207,16 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK212">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="AL212" t="s">
-        <v>1543</v>
+        <v>1245</v>
       </c>
       <c r="AM212">
         <v>1</v>
+      </c>
+      <c r="AN212" t="s">
+        <v>1565</v>
       </c>
     </row>
     <row r="213" spans="1:40" x14ac:dyDescent="0.25">
@@ -24305,10 +24308,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK213">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="AL213" t="s">
-        <v>1283</v>
+        <v>1543</v>
       </c>
       <c r="AM213">
         <v>1</v>
@@ -24403,10 +24406,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK214">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AL214" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="AM214">
         <v>1</v>
@@ -24498,16 +24501,13 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK215">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AL215" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="AM215">
         <v>1</v>
-      </c>
-      <c r="AN215" t="s">
-        <v>1565</v>
       </c>
     </row>
     <row r="216" spans="1:40" x14ac:dyDescent="0.25">
@@ -24599,16 +24599,16 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK216">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AL216" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="AM216">
         <v>1</v>
       </c>
       <c r="AN216" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="217" spans="1:40" x14ac:dyDescent="0.25">
@@ -24697,10 +24697,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK217">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AL217" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="AM217">
         <v>1</v>
@@ -24801,13 +24801,16 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK218">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AL218" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="AM218">
         <v>1</v>
+      </c>
+      <c r="AN218" t="s">
+        <v>1566</v>
       </c>
     </row>
     <row r="219" spans="1:40" x14ac:dyDescent="0.25">
@@ -24899,16 +24902,13 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK219">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="AL219" t="s">
-        <v>1431</v>
+        <v>1288</v>
       </c>
       <c r="AM219">
         <v>1</v>
-      </c>
-      <c r="AN219" t="s">
-        <v>1566</v>
       </c>
     </row>
     <row r="220" spans="1:40" x14ac:dyDescent="0.25">
@@ -25000,13 +25000,16 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK220">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="AL220" t="s">
-        <v>1289</v>
+        <v>1431</v>
       </c>
       <c r="AM220">
         <v>1</v>
+      </c>
+      <c r="AN220" t="s">
+        <v>1566</v>
       </c>
     </row>
     <row r="221" spans="1:40" x14ac:dyDescent="0.25">
@@ -25098,16 +25101,13 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK221">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="AL221" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="AM221">
         <v>1</v>
-      </c>
-      <c r="AN221" t="s">
-        <v>1565</v>
       </c>
     </row>
     <row r="222" spans="1:40" x14ac:dyDescent="0.25">
@@ -25196,16 +25196,16 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK222">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AL222" t="s">
-        <v>1437</v>
+        <v>1290</v>
       </c>
       <c r="AM222">
         <v>1</v>
       </c>
       <c r="AN222" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="223" spans="1:40" x14ac:dyDescent="0.25">
@@ -25300,10 +25300,10 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK223">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="AL223" t="s">
-        <v>1291</v>
+        <v>1437</v>
       </c>
       <c r="AM223">
         <v>1</v>
@@ -25398,13 +25398,16 @@
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="AK224">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="AL224" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="AM224">
         <v>1</v>
+      </c>
+      <c r="AN224" t="s">
+        <v>1566</v>
       </c>
     </row>
     <row r="225" spans="1:40" x14ac:dyDescent="0.25">
@@ -25496,10 +25499,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK225">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="AL225" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="AM225">
         <v>1</v>
@@ -25591,10 +25594,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK226">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="AL226" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="AM226">
         <v>1</v>
@@ -25686,10 +25689,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK227">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="AL227" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="AM227">
         <v>1</v>
@@ -25784,10 +25787,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK228">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="AL228" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="AM228">
         <v>1</v>
@@ -25894,10 +25897,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK229">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AL229" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="AM229">
         <v>1</v>
@@ -26001,10 +26004,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK230">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="AL230" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="AM230">
         <v>1</v>
@@ -26108,10 +26111,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK231">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AL231" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="AM231">
         <v>1</v>
@@ -26212,16 +26215,13 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK232">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="AL232" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
       <c r="AM232">
         <v>1</v>
-      </c>
-      <c r="AN232" t="s">
-        <v>1566</v>
       </c>
     </row>
     <row r="233" spans="1:40" x14ac:dyDescent="0.25">
@@ -26322,16 +26322,16 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK233">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="AL233" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="AM233">
         <v>1</v>
       </c>
       <c r="AN233" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="234" spans="1:40" x14ac:dyDescent="0.25">
@@ -26429,13 +26429,16 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK234">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="AL234" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="AM234">
         <v>1</v>
+      </c>
+      <c r="AN234" t="s">
+        <v>1567</v>
       </c>
     </row>
     <row r="235" spans="1:40" x14ac:dyDescent="0.25">
@@ -26536,16 +26539,13 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK235">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="AL235" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="AM235">
         <v>1</v>
-      </c>
-      <c r="AN235" t="s">
-        <v>1566</v>
       </c>
     </row>
     <row r="236" spans="1:40" x14ac:dyDescent="0.25">
@@ -26643,10 +26643,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK236">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="AL236" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="AM236">
         <v>1</v>
@@ -26753,10 +26753,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK237">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="AL237" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="AM237">
         <v>1</v>
@@ -26860,10 +26860,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK238">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="AL238" t="s">
-        <v>1546</v>
+        <v>1306</v>
       </c>
       <c r="AM238">
         <v>1</v>
@@ -26970,16 +26970,16 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK239">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="AL239" t="s">
-        <v>1307</v>
+        <v>1546</v>
       </c>
       <c r="AM239">
         <v>1</v>
       </c>
       <c r="AN239" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="240" spans="1:40" x14ac:dyDescent="0.25">
@@ -27080,13 +27080,16 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK240">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AL240" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="AM240">
         <v>1</v>
+      </c>
+      <c r="AN240" t="s">
+        <v>1565</v>
       </c>
     </row>
     <row r="241" spans="1:40" x14ac:dyDescent="0.25">
@@ -27184,10 +27187,10 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK241">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="AL241" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="AM241">
         <v>1</v>
@@ -27285,16 +27288,13 @@
         <v>4.7999999999999996E-3</v>
       </c>
       <c r="AK242">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="AL242" t="s">
-        <v>1547</v>
+        <v>1309</v>
       </c>
       <c r="AM242">
         <v>1</v>
-      </c>
-      <c r="AN242" t="s">
-        <v>1565</v>
       </c>
     </row>
     <row r="243" spans="1:40" x14ac:dyDescent="0.25">
@@ -27391,13 +27391,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK243">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="AL243" t="s">
-        <v>1548</v>
+        <v>1547</v>
       </c>
       <c r="AM243">
         <v>1</v>
+      </c>
+      <c r="AN243" t="s">
+        <v>1565</v>
       </c>
     </row>
     <row r="244" spans="1:40" x14ac:dyDescent="0.25">
@@ -27493,10 +27496,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK244">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AL244" t="s">
-        <v>1549</v>
+        <v>1548</v>
       </c>
       <c r="AM244">
         <v>1</v>
@@ -27592,16 +27595,13 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK245">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="AL245" t="s">
-        <v>1310</v>
+        <v>1549</v>
       </c>
       <c r="AM245">
         <v>1</v>
-      </c>
-      <c r="AN245" t="s">
-        <v>1566</v>
       </c>
     </row>
     <row r="246" spans="1:40" x14ac:dyDescent="0.25">
@@ -27699,16 +27699,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK246">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AL246" t="s">
-        <v>1550</v>
+        <v>1310</v>
       </c>
       <c r="AM246">
         <v>1</v>
       </c>
       <c r="AN246" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="247" spans="1:40" x14ac:dyDescent="0.25">
@@ -27806,16 +27806,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK247">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="AL247" t="s">
-        <v>1551</v>
+        <v>1550</v>
       </c>
       <c r="AM247">
         <v>1</v>
       </c>
       <c r="AN247" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="248" spans="1:40" x14ac:dyDescent="0.25">
@@ -27910,16 +27910,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK248">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="AL248" t="s">
-        <v>1311</v>
+        <v>1551</v>
       </c>
       <c r="AM248">
         <v>1</v>
       </c>
       <c r="AN248" t="s">
-        <v>1567</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="249" spans="1:40" x14ac:dyDescent="0.25">
@@ -28020,13 +28020,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK249">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="AL249" t="s">
-        <v>1455</v>
+        <v>1311</v>
       </c>
       <c r="AM249">
         <v>1</v>
+      </c>
+      <c r="AN249" t="s">
+        <v>1567</v>
       </c>
     </row>
     <row r="250" spans="1:40" x14ac:dyDescent="0.25">
@@ -28124,16 +28127,13 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK250">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AL250" t="s">
-        <v>1312</v>
+        <v>1455</v>
       </c>
       <c r="AM250">
         <v>1</v>
-      </c>
-      <c r="AN250" t="s">
-        <v>1567</v>
       </c>
     </row>
     <row r="251" spans="1:40" x14ac:dyDescent="0.25">
@@ -28231,13 +28231,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK251">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="AL251" t="s">
-        <v>1553</v>
+        <v>1312</v>
       </c>
       <c r="AM251">
         <v>1</v>
+      </c>
+      <c r="AN251" t="s">
+        <v>1567</v>
       </c>
     </row>
     <row r="252" spans="1:40" x14ac:dyDescent="0.25">
@@ -28332,16 +28335,13 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK252">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AL252" t="s">
-        <v>1313</v>
+        <v>1553</v>
       </c>
       <c r="AM252">
         <v>1</v>
-      </c>
-      <c r="AN252" t="s">
-        <v>1566</v>
       </c>
     </row>
     <row r="253" spans="1:40" x14ac:dyDescent="0.25">
@@ -28428,10 +28428,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK253">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="AL253" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="AM253">
         <v>1</v>
@@ -28530,10 +28530,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK254">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AL254" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="AM254">
         <v>1</v>
@@ -28635,13 +28635,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK255">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="AL255" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="AM255">
         <v>1</v>
+      </c>
+      <c r="AN255" t="s">
+        <v>1566</v>
       </c>
     </row>
     <row r="256" spans="1:40" x14ac:dyDescent="0.25">
@@ -28739,10 +28742,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK256">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="AL256" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="AM256">
         <v>1</v>
@@ -28843,10 +28846,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK257">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="AL257" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="AM257">
         <v>1</v>
@@ -28944,10 +28947,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK258">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="AL258" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="AM258">
         <v>1</v>
@@ -29048,10 +29051,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK259">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="AL259" t="s">
-        <v>1554</v>
+        <v>1319</v>
       </c>
       <c r="AM259">
         <v>1</v>
@@ -29152,16 +29155,13 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK260">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="AL260" t="s">
-        <v>1320</v>
+        <v>1554</v>
       </c>
       <c r="AM260">
         <v>1</v>
-      </c>
-      <c r="AN260" t="s">
-        <v>1566</v>
       </c>
     </row>
     <row r="261" spans="1:40" x14ac:dyDescent="0.25">
@@ -29256,16 +29256,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK261">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="AL261" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="AM261">
         <v>1</v>
       </c>
       <c r="AN261" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="262" spans="1:40" x14ac:dyDescent="0.25">
@@ -29363,16 +29363,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK262">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="AL262" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="AM262">
         <v>1</v>
       </c>
       <c r="AN262" t="s">
-        <v>1567</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="263" spans="1:40" x14ac:dyDescent="0.25">
@@ -29470,16 +29470,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK263">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="AL263" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="AM263">
         <v>1</v>
       </c>
       <c r="AN263" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="264" spans="1:40" x14ac:dyDescent="0.25">
@@ -29577,10 +29577,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK264">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="AL264" t="s">
-        <v>1555</v>
+        <v>1323</v>
       </c>
       <c r="AM264">
         <v>1</v>
@@ -29685,13 +29685,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK265">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="AL265" t="s">
-        <v>1324</v>
+        <v>1555</v>
       </c>
       <c r="AM265">
         <v>1</v>
+      </c>
+      <c r="AN265" t="s">
+        <v>1566</v>
       </c>
     </row>
     <row r="266" spans="1:40" x14ac:dyDescent="0.25">
@@ -29790,16 +29793,13 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK266">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="AL266" t="s">
-        <v>1469</v>
+        <v>1324</v>
       </c>
       <c r="AM266">
         <v>1</v>
-      </c>
-      <c r="AN266" t="s">
-        <v>1568</v>
       </c>
     </row>
     <row r="267" spans="1:40" x14ac:dyDescent="0.25">
@@ -29895,13 +29895,16 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK267">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="AL267" t="s">
-        <v>1325</v>
+        <v>1469</v>
       </c>
       <c r="AM267">
         <v>1</v>
+      </c>
+      <c r="AN267" t="s">
+        <v>1568</v>
       </c>
     </row>
     <row r="268" spans="1:40" x14ac:dyDescent="0.25">
@@ -29997,10 +30000,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK268">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AL268" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="AM268">
         <v>1</v>
@@ -30099,10 +30102,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK269">
-        <v>306</v>
+        <v>292</v>
       </c>
       <c r="AL269" t="s">
-        <v>1219</v>
+        <v>1326</v>
       </c>
       <c r="AM269">
         <v>1</v>
@@ -30204,7 +30207,7 @@
         <v>307</v>
       </c>
       <c r="AL270" t="s">
-        <v>1254</v>
+        <v>1219</v>
       </c>
       <c r="AM270">
         <v>1</v>
@@ -30306,10 +30309,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK271">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="AL271" t="s">
-        <v>1252</v>
+        <v>1254</v>
       </c>
       <c r="AM271">
         <v>1</v>
@@ -30399,10 +30402,10 @@
         <v>5.4999999999999997E-3</v>
       </c>
       <c r="AK272">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="AL272" t="s">
-        <v>1330</v>
+        <v>1252</v>
       </c>
       <c r="AM272">
         <v>1</v>
@@ -30492,7 +30495,7 @@
         <v>313</v>
       </c>
       <c r="AL273" t="s">
-        <v>1278</v>
+        <v>1330</v>
       </c>
       <c r="AM273">
         <v>1</v>
@@ -30585,7 +30588,7 @@
         <v>314</v>
       </c>
       <c r="AL274" t="s">
-        <v>1221</v>
+        <v>1278</v>
       </c>
       <c r="AM274">
         <v>1</v>
@@ -30675,7 +30678,7 @@
         <v>315</v>
       </c>
       <c r="AL275" t="s">
-        <v>1262</v>
+        <v>1221</v>
       </c>
       <c r="AM275">
         <v>1</v>
@@ -30774,7 +30777,7 @@
         <v>316</v>
       </c>
       <c r="AL276" t="s">
-        <v>1232</v>
+        <v>1262</v>
       </c>
       <c r="AM276">
         <v>1</v>
@@ -30876,7 +30879,7 @@
         <v>317</v>
       </c>
       <c r="AL277" t="s">
-        <v>1328</v>
+        <v>1232</v>
       </c>
       <c r="AM277">
         <v>1</v>
@@ -30975,7 +30978,7 @@
         <v>318</v>
       </c>
       <c r="AL278" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="AM278">
         <v>1</v>
@@ -31077,7 +31080,7 @@
         <v>319</v>
       </c>
       <c r="AL279" t="s">
-        <v>1222</v>
+        <v>1329</v>
       </c>
       <c r="AM279">
         <v>1</v>
@@ -31176,7 +31179,7 @@
         <v>320</v>
       </c>
       <c r="AL280" t="s">
-        <v>1414</v>
+        <v>1222</v>
       </c>
       <c r="AM280">
         <v>1</v>
@@ -31275,7 +31278,7 @@
         <v>321</v>
       </c>
       <c r="AL281" t="s">
-        <v>1419</v>
+        <v>1414</v>
       </c>
       <c r="AM281">
         <v>1</v>
@@ -31377,7 +31380,7 @@
         <v>322</v>
       </c>
       <c r="AL282" t="s">
-        <v>1372</v>
+        <v>1419</v>
       </c>
       <c r="AM282">
         <v>1</v>
@@ -31476,7 +31479,7 @@
         <v>323</v>
       </c>
       <c r="AL283" t="s">
-        <v>1363</v>
+        <v>1372</v>
       </c>
       <c r="AM283">
         <v>1</v>
@@ -31577,7 +31580,7 @@
         <v>324</v>
       </c>
       <c r="AL284" t="s">
-        <v>1374</v>
+        <v>1363</v>
       </c>
       <c r="AM284">
         <v>1</v>
@@ -31675,7 +31678,7 @@
         <v>325</v>
       </c>
       <c r="AL285" t="s">
-        <v>1345</v>
+        <v>1374</v>
       </c>
       <c r="AM285">
         <v>1</v>
@@ -31774,7 +31777,7 @@
         <v>326</v>
       </c>
       <c r="AL286" t="s">
-        <v>1405</v>
+        <v>1345</v>
       </c>
       <c r="AM286">
         <v>1</v>
@@ -31870,7 +31873,7 @@
         <v>327</v>
       </c>
       <c r="AL287" t="s">
-        <v>1368</v>
+        <v>1405</v>
       </c>
       <c r="AM287">
         <v>1</v>
@@ -31969,7 +31972,7 @@
         <v>328</v>
       </c>
       <c r="AL288" t="s">
-        <v>1346</v>
+        <v>1368</v>
       </c>
       <c r="AM288">
         <v>1</v>
@@ -32068,7 +32071,7 @@
         <v>329</v>
       </c>
       <c r="AL289" t="s">
-        <v>1360</v>
+        <v>1346</v>
       </c>
       <c r="AM289">
         <v>1</v>
@@ -32164,7 +32167,7 @@
         <v>330</v>
       </c>
       <c r="AL290" t="s">
-        <v>1370</v>
+        <v>1360</v>
       </c>
       <c r="AM290">
         <v>1</v>
@@ -32263,7 +32266,7 @@
         <v>331</v>
       </c>
       <c r="AL291" t="s">
-        <v>1378</v>
+        <v>1370</v>
       </c>
       <c r="AM291">
         <v>1</v>
@@ -32359,7 +32362,7 @@
         <v>332</v>
       </c>
       <c r="AL292" t="s">
-        <v>1354</v>
+        <v>1378</v>
       </c>
       <c r="AM292">
         <v>1</v>
@@ -32455,10 +32458,10 @@
         <v>6.1999999999999998E-3</v>
       </c>
       <c r="AK293">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="AL293" t="s">
-        <v>1347</v>
+        <v>1354</v>
       </c>
       <c r="AM293">
         <v>1</v>
@@ -32554,7 +32557,7 @@
         <v>335</v>
       </c>
       <c r="AL294" t="s">
-        <v>1341</v>
+        <v>1347</v>
       </c>
       <c r="AM294">
         <v>1</v>
@@ -32650,7 +32653,7 @@
         <v>336</v>
       </c>
       <c r="AL295" t="s">
-        <v>1344</v>
+        <v>1341</v>
       </c>
       <c r="AM295">
         <v>1</v>
@@ -32754,7 +32757,7 @@
         <v>337</v>
       </c>
       <c r="AL296" t="s">
-        <v>1364</v>
+        <v>1344</v>
       </c>
       <c r="AM296">
         <v>1</v>
@@ -32855,7 +32858,7 @@
         <v>338</v>
       </c>
       <c r="AL297" t="s">
-        <v>1357</v>
+        <v>1364</v>
       </c>
       <c r="AM297">
         <v>1</v>
@@ -32959,7 +32962,7 @@
         <v>339</v>
       </c>
       <c r="AL298" t="s">
-        <v>1349</v>
+        <v>1357</v>
       </c>
       <c r="AM298">
         <v>1</v>
@@ -33063,7 +33066,7 @@
         <v>340</v>
       </c>
       <c r="AL299" t="s">
-        <v>1253</v>
+        <v>1349</v>
       </c>
       <c r="AM299">
         <v>1</v>
@@ -33164,7 +33167,7 @@
         <v>341</v>
       </c>
       <c r="AL300" t="s">
-        <v>1242</v>
+        <v>1253</v>
       </c>
       <c r="AM300">
         <v>1</v>
@@ -33268,7 +33271,7 @@
         <v>342</v>
       </c>
       <c r="AL301" t="s">
-        <v>1426</v>
+        <v>1242</v>
       </c>
       <c r="AM301">
         <v>1</v>
@@ -33366,10 +33369,10 @@
         <v>6.7999999999999996E-3</v>
       </c>
       <c r="AK302">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="AL302" t="s">
-        <v>1218</v>
+        <v>1426</v>
       </c>
       <c r="AM302">
         <v>1</v>
@@ -33476,7 +33479,7 @@
         <v>345</v>
       </c>
       <c r="AL303" t="s">
-        <v>1279</v>
+        <v>1218</v>
       </c>
       <c r="AM303">
         <v>1</v>
@@ -33580,7 +33583,7 @@
         <v>346</v>
       </c>
       <c r="AL304" t="s">
-        <v>1259</v>
+        <v>1279</v>
       </c>
       <c r="AM304">
         <v>1</v>
@@ -33682,7 +33685,7 @@
         <v>347</v>
       </c>
       <c r="AL305" t="s">
-        <v>1557</v>
+        <v>1259</v>
       </c>
       <c r="AM305">
         <v>1</v>
@@ -33784,7 +33787,7 @@
         <v>348</v>
       </c>
       <c r="AL306" t="s">
-        <v>1379</v>
+        <v>1557</v>
       </c>
       <c r="AM306">
         <v>1</v>
@@ -33886,7 +33889,7 @@
         <v>349</v>
       </c>
       <c r="AL307" t="s">
-        <v>1558</v>
+        <v>1379</v>
       </c>
       <c r="AM307">
         <v>1</v>
@@ -33988,7 +33991,7 @@
         <v>350</v>
       </c>
       <c r="AL308" t="s">
-        <v>1559</v>
+        <v>1558</v>
       </c>
       <c r="AM308">
         <v>1</v>
@@ -34090,7 +34093,7 @@
         <v>351</v>
       </c>
       <c r="AL309" t="s">
-        <v>1560</v>
+        <v>1559</v>
       </c>
       <c r="AM309">
         <v>1</v>
@@ -34189,7 +34192,7 @@
         <v>352</v>
       </c>
       <c r="AL310" t="s">
-        <v>1561</v>
+        <v>1560</v>
       </c>
       <c r="AM310">
         <v>1</v>
@@ -34293,7 +34296,7 @@
         <v>353</v>
       </c>
       <c r="AL311" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="AM311">
         <v>1</v>
@@ -34394,10 +34397,10 @@
         <v>7.4999999999999997E-3</v>
       </c>
       <c r="AK312">
-        <v>364</v>
+        <v>354</v>
       </c>
       <c r="AL312" t="s">
-        <v>1427</v>
+        <v>1562</v>
       </c>
       <c r="AM312">
         <v>1</v>
@@ -34495,7 +34498,7 @@
         <v>365</v>
       </c>
       <c r="AL313" t="s">
-        <v>1404</v>
+        <v>1427</v>
       </c>
       <c r="AM313">
         <v>1</v>
@@ -34593,10 +34596,10 @@
         <v>7.4999999999999997E-3</v>
       </c>
       <c r="AK314">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="AL314" t="s">
-        <v>1425</v>
+        <v>1404</v>
       </c>
       <c r="AM314">
         <v>1</v>
@@ -34691,10 +34694,10 @@
         <v>7.4999999999999997E-3</v>
       </c>
       <c r="AK315">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="AL315" t="s">
-        <v>1473</v>
+        <v>1425</v>
       </c>
       <c r="AM315">
         <v>1</v>
@@ -34795,7 +34798,7 @@
         <v>370</v>
       </c>
       <c r="AL316" t="s">
-        <v>1392</v>
+        <v>1473</v>
       </c>
       <c r="AM316">
         <v>1</v>
@@ -34896,7 +34899,7 @@
         <v>371</v>
       </c>
       <c r="AL317" t="s">
-        <v>1402</v>
+        <v>1392</v>
       </c>
       <c r="AM317">
         <v>1</v>
@@ -34994,7 +34997,7 @@
         <v>372</v>
       </c>
       <c r="AL318" t="s">
-        <v>1384</v>
+        <v>1402</v>
       </c>
       <c r="AM318">
         <v>1</v>
@@ -35093,7 +35096,7 @@
         <v>373</v>
       </c>
       <c r="AL319" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
       <c r="AM319">
         <v>1</v>
@@ -35192,7 +35195,7 @@
         <v>374</v>
       </c>
       <c r="AL320" t="s">
-        <v>1420</v>
+        <v>1386</v>
       </c>
       <c r="AM320">
         <v>1</v>
@@ -35288,7 +35291,7 @@
         <v>375</v>
       </c>
       <c r="AL321" t="s">
-        <v>1393</v>
+        <v>1420</v>
       </c>
       <c r="AM321">
         <v>1</v>
@@ -35387,7 +35390,7 @@
         <v>376</v>
       </c>
       <c r="AL322" t="s">
-        <v>1389</v>
+        <v>1393</v>
       </c>
       <c r="AM322">
         <v>1</v>
@@ -35483,7 +35486,7 @@
         <v>377</v>
       </c>
       <c r="AL323" t="s">
-        <v>1421</v>
+        <v>1389</v>
       </c>
       <c r="AM323">
         <v>1</v>
@@ -35582,7 +35585,7 @@
         <v>378</v>
       </c>
       <c r="AL324" t="s">
-        <v>1376</v>
+        <v>1421</v>
       </c>
       <c r="AM324">
         <v>1</v>
@@ -35678,7 +35681,7 @@
         <v>379</v>
       </c>
       <c r="AL325" t="s">
-        <v>1391</v>
+        <v>1376</v>
       </c>
       <c r="AM325">
         <v>1</v>
@@ -35748,7 +35751,7 @@
         <v>380</v>
       </c>
       <c r="AL326" t="s">
-        <v>1382</v>
+        <v>1391</v>
       </c>
       <c r="AM326">
         <v>1</v>
@@ -35821,7 +35824,7 @@
         <v>381</v>
       </c>
       <c r="AL327" t="s">
-        <v>1429</v>
+        <v>1382</v>
       </c>
       <c r="AM327">
         <v>1</v>
@@ -35891,7 +35894,7 @@
         <v>1002</v>
       </c>
       <c r="AL328" t="s">
-        <v>1380</v>
+        <v>1429</v>
       </c>
       <c r="AM328">
         <v>1</v>
@@ -35956,7 +35959,7 @@
         <v>1022</v>
       </c>
       <c r="AL329" t="s">
-        <v>1409</v>
+        <v>1380</v>
       </c>
       <c r="AM329">
         <v>1</v>
@@ -36021,7 +36024,7 @@
         <v>1022</v>
       </c>
       <c r="AL330" t="s">
-        <v>1411</v>
+        <v>1409</v>
       </c>
       <c r="AM330">
         <v>1</v>
@@ -36086,7 +36089,7 @@
         <v>1002</v>
       </c>
       <c r="AL331" t="s">
-        <v>1390</v>
+        <v>1411</v>
       </c>
       <c r="AM331">
         <v>1</v>
@@ -36153,14 +36156,11 @@
       <c r="X332" s="24" t="s">
         <v>1023</v>
       </c>
-      <c r="AK332">
-        <v>9</v>
-      </c>
       <c r="AL332" t="s">
-        <v>1521</v>
+        <v>1390</v>
       </c>
       <c r="AM332">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="333" spans="1:39" x14ac:dyDescent="0.25">
@@ -36225,10 +36225,10 @@
         <v>1023</v>
       </c>
       <c r="AK333">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="AL333" t="s">
-        <v>1217</v>
+        <v>1521</v>
       </c>
       <c r="AM333">
         <v>2</v>
@@ -36290,10 +36290,10 @@
         <v>1022</v>
       </c>
       <c r="AK334">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="AL334" t="s">
-        <v>1239</v>
+        <v>1217</v>
       </c>
       <c r="AM334">
         <v>2</v>
@@ -36354,10 +36354,10 @@
         <v>40</v>
       </c>
       <c r="AK335">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="AL335" t="s">
-        <v>1359</v>
+        <v>1239</v>
       </c>
       <c r="AM335">
         <v>2</v>
@@ -36424,10 +36424,10 @@
         <v>1331</v>
       </c>
       <c r="AK336">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="AL336" t="s">
-        <v>1422</v>
+        <v>1359</v>
       </c>
       <c r="AM336">
         <v>2</v>
@@ -36494,10 +36494,10 @@
         <v>1336</v>
       </c>
       <c r="AK337">
-        <v>305</v>
+        <v>69</v>
       </c>
       <c r="AL337" t="s">
-        <v>1273</v>
+        <v>1422</v>
       </c>
       <c r="AM337">
         <v>2</v>
@@ -36567,10 +36567,10 @@
         <v>1334</v>
       </c>
       <c r="AK338">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="AL338" t="s">
-        <v>1265</v>
+        <v>1273</v>
       </c>
       <c r="AM338">
         <v>2</v>
@@ -36640,10 +36640,10 @@
         <v>1340</v>
       </c>
       <c r="AK339">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="AL339" t="s">
-        <v>1277</v>
+        <v>1265</v>
       </c>
       <c r="AM339">
         <v>2</v>
@@ -36722,13 +36722,13 @@
         <v>1335</v>
       </c>
       <c r="AK340">
-        <v>33</v>
+        <v>312</v>
       </c>
       <c r="AL340" t="s">
-        <v>1226</v>
+        <v>1277</v>
       </c>
       <c r="AM340">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="341" spans="1:39" x14ac:dyDescent="0.25">
@@ -36798,10 +36798,10 @@
         <v>1516</v>
       </c>
       <c r="AK341">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="AL341" t="s">
-        <v>798</v>
+        <v>1226</v>
       </c>
       <c r="AM341">
         <v>3</v>
@@ -36868,10 +36868,10 @@
         <v>0</v>
       </c>
       <c r="AK342">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AL342" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="AM342">
         <v>3</v>
@@ -36950,10 +36950,10 @@
         <v>1650</v>
       </c>
       <c r="AK343">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="AL343" t="s">
-        <v>1362</v>
+        <v>799</v>
       </c>
       <c r="AM343">
         <v>3</v>
@@ -37020,10 +37020,10 @@
         <v>4</v>
       </c>
       <c r="AK344">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="AL344" t="s">
-        <v>1356</v>
+        <v>1362</v>
       </c>
       <c r="AM344">
         <v>3</v>
@@ -37088,10 +37088,10 @@
         <v>20</v>
       </c>
       <c r="AK345">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="AL345" t="s">
-        <v>1260</v>
+        <v>1356</v>
       </c>
       <c r="AM345">
         <v>3</v>
@@ -37149,10 +37149,10 @@
         <v>Soldrota-E</v>
       </c>
       <c r="AK346">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AL346" t="s">
-        <v>1412</v>
+        <v>1260</v>
       </c>
       <c r="AM346">
         <v>3</v>
@@ -37211,10 +37211,10 @@
         <v>35</v>
       </c>
       <c r="AK347">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="AL347" t="s">
-        <v>1227</v>
+        <v>1412</v>
       </c>
       <c r="AM347">
         <v>3</v>
@@ -37273,10 +37273,10 @@
         <v>55</v>
       </c>
       <c r="AK348">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="AL348" t="s">
-        <v>1282</v>
+        <v>1227</v>
       </c>
       <c r="AM348">
         <v>3</v>
@@ -37332,10 +37332,10 @@
         <v>Blastflames-E</v>
       </c>
       <c r="AK349">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="AL349" t="s">
-        <v>1249</v>
+        <v>1282</v>
       </c>
       <c r="AM349">
         <v>3</v>
@@ -37394,10 +37394,10 @@
         <v>22</v>
       </c>
       <c r="AK350">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="AL350" t="s">
-        <v>1276</v>
+        <v>1249</v>
       </c>
       <c r="AM350">
         <v>3</v>
@@ -37456,10 +37456,10 @@
         <v>796</v>
       </c>
       <c r="AK351">
-        <v>302</v>
+        <v>82</v>
       </c>
       <c r="AL351" t="s">
-        <v>1229</v>
+        <v>1276</v>
       </c>
       <c r="AM351">
         <v>3</v>
@@ -37518,7 +37518,7 @@
         <v>303</v>
       </c>
       <c r="AL352" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="AM352">
         <v>3</v>
@@ -37580,7 +37580,7 @@
         <v>304</v>
       </c>
       <c r="AL353" t="s">
-        <v>1264</v>
+        <v>1230</v>
       </c>
       <c r="AM353">
         <v>3</v>
@@ -37639,13 +37639,13 @@
         <v>20</v>
       </c>
       <c r="AK354">
-        <v>2</v>
+        <v>305</v>
       </c>
       <c r="AL354" t="s">
-        <v>1244</v>
+        <v>1264</v>
       </c>
       <c r="AM354">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="355" spans="1:39" x14ac:dyDescent="0.25">
@@ -37701,10 +37701,10 @@
         <v>Gyarados-E</v>
       </c>
       <c r="AK355">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="AL355" t="s">
-        <v>1220</v>
+        <v>1244</v>
       </c>
       <c r="AM355">
         <v>4</v>
@@ -37762,10 +37762,10 @@
         <v>Shockfang</v>
       </c>
       <c r="AK356">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="AL356" t="s">
-        <v>1237</v>
+        <v>1220</v>
       </c>
       <c r="AM356">
         <v>4</v>
@@ -37826,10 +37826,10 @@
         <v>40</v>
       </c>
       <c r="AK357">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="AL357" t="s">
-        <v>1375</v>
+        <v>1237</v>
       </c>
       <c r="AM357">
         <v>4</v>
@@ -37887,10 +37887,10 @@
         <v>Nightrex</v>
       </c>
       <c r="AK358">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="AL358" t="s">
-        <v>1215</v>
+        <v>1375</v>
       </c>
       <c r="AM358">
         <v>4</v>
@@ -37951,10 +37951,10 @@
         <v>40</v>
       </c>
       <c r="AK359">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="AL359" t="s">
-        <v>1223</v>
+        <v>1215</v>
       </c>
       <c r="AM359">
         <v>4</v>
@@ -38010,10 +38010,10 @@
         <v>Durfish-S</v>
       </c>
       <c r="AK360">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AL360" t="s">
-        <v>1248</v>
+        <v>1223</v>
       </c>
       <c r="AM360">
         <v>4</v>
@@ -38072,10 +38072,10 @@
         <v>794</v>
       </c>
       <c r="AK361">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AL361" t="s">
-        <v>1355</v>
+        <v>1248</v>
       </c>
       <c r="AM361">
         <v>4</v>
@@ -38130,10 +38130,10 @@
         <v>Wormite-S</v>
       </c>
       <c r="AK362">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="AL362" t="s">
-        <v>1361</v>
+        <v>1355</v>
       </c>
       <c r="AM362">
         <v>4</v>
@@ -38191,10 +38191,10 @@
         <v>20</v>
       </c>
       <c r="AK363">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="AL363" t="s">
-        <v>1350</v>
+        <v>1361</v>
       </c>
       <c r="AM363">
         <v>4</v>
@@ -38251,8 +38251,11 @@
       <c r="R364">
         <v>45</v>
       </c>
+      <c r="AK364">
+        <v>75</v>
+      </c>
       <c r="AL364" t="s">
-        <v>1423</v>
+        <v>1350</v>
       </c>
       <c r="AM364">
         <v>4</v>
@@ -38306,14 +38309,11 @@
         <f t="shared" si="20"/>
         <v>Cluuz-S</v>
       </c>
-      <c r="AK365">
-        <v>1</v>
-      </c>
       <c r="AL365" t="s">
-        <v>1267</v>
+        <v>1423</v>
       </c>
       <c r="AM365">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="366" spans="1:39" x14ac:dyDescent="0.25">
@@ -38368,10 +38368,10 @@
         <v>794</v>
       </c>
       <c r="AK366">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="AL366" t="s">
-        <v>1263</v>
+        <v>1267</v>
       </c>
       <c r="AM366">
         <v>5</v>
@@ -38429,10 +38429,10 @@
         <v>788</v>
       </c>
       <c r="AK367">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="AL367" t="s">
-        <v>1373</v>
+        <v>1263</v>
       </c>
       <c r="AM367">
         <v>5</v>
@@ -38493,10 +38493,10 @@
         <v>16</v>
       </c>
       <c r="AK368">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="AL368" t="s">
-        <v>1231</v>
+        <v>1373</v>
       </c>
       <c r="AM368">
         <v>5</v>
@@ -38557,10 +38557,10 @@
         <v>36</v>
       </c>
       <c r="AK369">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="AL369" t="s">
-        <v>1225</v>
+        <v>1231</v>
       </c>
       <c r="AM369">
         <v>5</v>
@@ -38618,10 +38618,10 @@
         <v>Pyrator-S</v>
       </c>
       <c r="AK370">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="AL370" t="s">
-        <v>1352</v>
+        <v>1225</v>
       </c>
       <c r="AM370">
         <v>5</v>
@@ -38682,10 +38682,10 @@
         <v>32</v>
       </c>
       <c r="AK371">
-        <v>162</v>
+        <v>79</v>
       </c>
       <c r="AL371" t="s">
-        <v>1488</v>
+        <v>1352</v>
       </c>
       <c r="AM371">
         <v>5</v>
@@ -38743,10 +38743,10 @@
         <v>Arbok-S</v>
       </c>
       <c r="AK372">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AL372" t="s">
-        <v>1489</v>
+        <v>1488</v>
       </c>
       <c r="AM372">
         <v>5</v>
@@ -38802,10 +38802,10 @@
         <v>862</v>
       </c>
       <c r="AK373">
-        <v>310</v>
+        <v>163</v>
       </c>
       <c r="AL373" t="s">
-        <v>1261</v>
+        <v>1489</v>
       </c>
       <c r="AM373">
         <v>5</v>
@@ -38860,8 +38860,11 @@
       <c r="R374" t="s">
         <v>866</v>
       </c>
+      <c r="AK374">
+        <v>311</v>
+      </c>
       <c r="AL374" t="s">
-        <v>1424</v>
+        <v>1261</v>
       </c>
       <c r="AM374">
         <v>5</v>
@@ -38916,14 +38919,11 @@
       <c r="R375" t="s">
         <v>863</v>
       </c>
-      <c r="AK375">
-        <v>30</v>
-      </c>
       <c r="AL375" t="s">
-        <v>1241</v>
+        <v>1424</v>
       </c>
       <c r="AM375">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="376" spans="1:40" x14ac:dyDescent="0.25">
@@ -38976,10 +38976,10 @@
         <v>819</v>
       </c>
       <c r="AK376">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="AL376" t="s">
-        <v>1251</v>
+        <v>1241</v>
       </c>
       <c r="AM376">
         <v>6</v>
@@ -39035,10 +39035,10 @@
         <v>863</v>
       </c>
       <c r="AK377">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="AL377" t="s">
-        <v>1234</v>
+        <v>1251</v>
       </c>
       <c r="AM377">
         <v>6</v>
@@ -39094,10 +39094,10 @@
         <v>849</v>
       </c>
       <c r="AK378">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="AL378" t="s">
-        <v>1247</v>
+        <v>1234</v>
       </c>
       <c r="AM378">
         <v>6</v>
@@ -39153,10 +39153,10 @@
         <v>851</v>
       </c>
       <c r="AK379">
-        <v>172</v>
+        <v>56</v>
       </c>
       <c r="AL379" t="s">
-        <v>907</v>
+        <v>1247</v>
       </c>
       <c r="AM379">
         <v>6</v>
@@ -39212,10 +39212,10 @@
         <v>864</v>
       </c>
       <c r="AK380">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AL380" t="s">
-        <v>1019</v>
+        <v>907</v>
       </c>
       <c r="AM380">
         <v>6</v>
@@ -39271,10 +39271,10 @@
         <v>1092</v>
       </c>
       <c r="AK381">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="AL381" t="s">
-        <v>1497</v>
+        <v>1019</v>
       </c>
       <c r="AM381">
         <v>6</v>
@@ -39323,16 +39323,13 @@
         <v>Kissyfishy-D</v>
       </c>
       <c r="AK382">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="AL382" t="s">
-        <v>1539</v>
+        <v>1497</v>
       </c>
       <c r="AM382">
         <v>6</v>
-      </c>
-      <c r="AN382" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="383" spans="1:40" x14ac:dyDescent="0.25">
@@ -39380,10 +39377,10 @@
         <v>623</v>
       </c>
       <c r="AK383">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AL383" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="AM383">
         <v>6</v>
@@ -39437,10 +39434,10 @@
         <v>623</v>
       </c>
       <c r="AK384">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AL384" t="s">
-        <v>1541</v>
+        <v>1540</v>
       </c>
       <c r="AM384">
         <v>6</v>
@@ -39494,10 +39491,10 @@
         <v>623</v>
       </c>
       <c r="AK385">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="AL385" t="s">
-        <v>1542</v>
+        <v>1541</v>
       </c>
       <c r="AM385">
         <v>6</v>
@@ -39542,13 +39539,16 @@
         <v>350</v>
       </c>
       <c r="AK386">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="AL386" t="s">
-        <v>1491</v>
+        <v>1542</v>
       </c>
       <c r="AM386">
-        <v>7</v>
+        <v>6</v>
+      </c>
+      <c r="AN386" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="387" spans="1:40" x14ac:dyDescent="0.25">
@@ -39587,10 +39587,10 @@
         <v>525</v>
       </c>
       <c r="AK387">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AL387" t="s">
-        <v>1492</v>
+        <v>1491</v>
       </c>
       <c r="AM387">
         <v>7</v>
@@ -39632,10 +39632,10 @@
         <v>310</v>
       </c>
       <c r="AK388">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AL388" t="s">
-        <v>1493</v>
+        <v>1492</v>
       </c>
       <c r="AM388">
         <v>7</v>
@@ -39677,10 +39677,10 @@
         <v>400</v>
       </c>
       <c r="AK389">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AL389" t="s">
-        <v>1494</v>
+        <v>1493</v>
       </c>
       <c r="AM389">
         <v>7</v>
@@ -39722,10 +39722,10 @@
         <v>500</v>
       </c>
       <c r="AK390">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="AL390" t="s">
-        <v>1498</v>
+        <v>1494</v>
       </c>
       <c r="AM390">
         <v>7</v>
@@ -39767,13 +39767,13 @@
         <v>500</v>
       </c>
       <c r="AK391">
-        <v>27</v>
+        <v>179</v>
       </c>
       <c r="AL391" t="s">
-        <v>1280</v>
+        <v>1498</v>
       </c>
       <c r="AM391">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="392" spans="1:40" x14ac:dyDescent="0.25">
@@ -39812,10 +39812,10 @@
         <v>430</v>
       </c>
       <c r="AK392">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="AL392" t="s">
-        <v>1235</v>
+        <v>1280</v>
       </c>
       <c r="AM392">
         <v>8</v>
@@ -39857,10 +39857,10 @@
         <v>510</v>
       </c>
       <c r="AK393">
-        <v>174</v>
+        <v>41</v>
       </c>
       <c r="AL393" t="s">
-        <v>1495</v>
+        <v>1235</v>
       </c>
       <c r="AM393">
         <v>8</v>
@@ -39902,10 +39902,10 @@
         <v>510</v>
       </c>
       <c r="AK394">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="AL394" t="s">
-        <v>1499</v>
+        <v>1495</v>
       </c>
       <c r="AM394">
         <v>8</v>
@@ -39947,16 +39947,13 @@
         <v>510</v>
       </c>
       <c r="AK395">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AL395" t="s">
-        <v>1500</v>
+        <v>1499</v>
       </c>
       <c r="AM395">
         <v>8</v>
-      </c>
-      <c r="AN395" t="s">
-        <v>1563</v>
       </c>
     </row>
     <row r="396" spans="1:40" x14ac:dyDescent="0.25">
@@ -39995,13 +39992,16 @@
         <v>290</v>
       </c>
       <c r="AK396">
-        <v>36</v>
+        <v>181</v>
       </c>
       <c r="AL396" t="s">
-        <v>1240</v>
+        <v>1500</v>
       </c>
       <c r="AM396">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="AN396" t="s">
+        <v>1563</v>
       </c>
     </row>
     <row r="397" spans="1:40" x14ac:dyDescent="0.25">
@@ -40040,10 +40040,10 @@
         <v>370</v>
       </c>
       <c r="AK397">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="AL397" t="s">
-        <v>1214</v>
+        <v>1240</v>
       </c>
       <c r="AM397">
         <v>9</v>
@@ -40085,10 +40085,10 @@
         <v>490</v>
       </c>
       <c r="AK398">
-        <v>164</v>
+        <v>60</v>
       </c>
       <c r="AL398" t="s">
-        <v>901</v>
+        <v>1214</v>
       </c>
       <c r="AM398">
         <v>9</v>
@@ -40130,10 +40130,10 @@
         <v>290</v>
       </c>
       <c r="AK399">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AL399" t="s">
-        <v>908</v>
+        <v>901</v>
       </c>
       <c r="AM399">
         <v>9</v>
@@ -40175,10 +40175,10 @@
         <v>370</v>
       </c>
       <c r="AK400">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AL400" t="s">
-        <v>1258</v>
+        <v>908</v>
       </c>
       <c r="AM400">
         <v>9</v>
@@ -40220,10 +40220,10 @@
         <v>490</v>
       </c>
       <c r="AK401">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="AL401" t="s">
-        <v>1490</v>
+        <v>1258</v>
       </c>
       <c r="AM401">
         <v>9</v>
@@ -40265,10 +40265,10 @@
         <v>458</v>
       </c>
       <c r="AK402">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="AL402" t="s">
-        <v>1017</v>
+        <v>1490</v>
       </c>
       <c r="AM402">
         <v>9</v>
@@ -40310,10 +40310,10 @@
         <v>535</v>
       </c>
       <c r="AK403">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AL403" t="s">
-        <v>1496</v>
+        <v>1017</v>
       </c>
       <c r="AM403">
         <v>9</v>
@@ -40355,13 +40355,13 @@
         <v>312</v>
       </c>
       <c r="AK404">
-        <v>26</v>
+        <v>177</v>
       </c>
       <c r="AL404" t="s">
-        <v>1268</v>
+        <v>1496</v>
       </c>
       <c r="AM404">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="405" spans="1:39" x14ac:dyDescent="0.25">
@@ -40400,10 +40400,10 @@
         <v>487</v>
       </c>
       <c r="AK405">
-        <v>161</v>
+        <v>26</v>
       </c>
       <c r="AL405" t="s">
-        <v>1216</v>
+        <v>1268</v>
       </c>
       <c r="AM405">
         <v>10</v>
@@ -40445,10 +40445,10 @@
         <v>332</v>
       </c>
       <c r="AK406">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="AL406" t="s">
-        <v>1018</v>
+        <v>1216</v>
       </c>
       <c r="AM406">
         <v>10</v>
@@ -40490,13 +40490,13 @@
         <v>497</v>
       </c>
       <c r="AK407">
-        <v>29</v>
+        <v>175</v>
       </c>
       <c r="AL407" t="s">
-        <v>1256</v>
+        <v>1018</v>
       </c>
       <c r="AM407">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="408" spans="1:39" x14ac:dyDescent="0.25">
@@ -40535,10 +40535,10 @@
         <v>410</v>
       </c>
       <c r="AK408">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="AL408" t="s">
-        <v>1269</v>
+        <v>1256</v>
       </c>
       <c r="AM408">
         <v>12</v>
@@ -40579,8 +40579,11 @@
       <c r="K409">
         <v>570</v>
       </c>
+      <c r="AK409">
+        <v>44</v>
+      </c>
       <c r="AL409" t="s">
-        <v>1342</v>
+        <v>1269</v>
       </c>
       <c r="AM409">
         <v>12</v>
@@ -40627,14 +40630,11 @@
       <c r="N410" t="s">
         <v>1191</v>
       </c>
-      <c r="AK410">
-        <v>3</v>
-      </c>
       <c r="AL410" t="s">
-        <v>1327</v>
+        <v>1342</v>
       </c>
       <c r="AM410">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="411" spans="1:39" x14ac:dyDescent="0.25">
@@ -40679,10 +40679,10 @@
         <v>1191</v>
       </c>
       <c r="AK411">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="AL411" t="s">
-        <v>1257</v>
+        <v>1327</v>
       </c>
       <c r="AM411">
         <v>13</v>
@@ -40723,11 +40723,14 @@
       <c r="K412">
         <v>335</v>
       </c>
+      <c r="AK412">
+        <v>39</v>
+      </c>
       <c r="AL412" t="s">
-        <v>1371</v>
+        <v>1257</v>
       </c>
       <c r="AM412">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="413" spans="1:39" x14ac:dyDescent="0.25">
@@ -40766,7 +40769,7 @@
         <v>485</v>
       </c>
       <c r="AL413" t="s">
-        <v>1343</v>
+        <v>1371</v>
       </c>
       <c r="AM413">
         <v>14</v>
@@ -40807,14 +40810,11 @@
       <c r="K414">
         <v>195</v>
       </c>
-      <c r="AK414">
-        <v>42</v>
-      </c>
       <c r="AL414" t="s">
-        <v>1255</v>
+        <v>1343</v>
       </c>
       <c r="AM414">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="415" spans="1:39" x14ac:dyDescent="0.25">
@@ -40853,13 +40853,13 @@
         <v>205</v>
       </c>
       <c r="AK415">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="AL415" t="s">
-        <v>1243</v>
+        <v>1255</v>
       </c>
       <c r="AM415">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="416" spans="1:39" x14ac:dyDescent="0.25">
@@ -40897,8 +40897,11 @@
       <c r="K416">
         <v>400</v>
       </c>
+      <c r="AK416">
+        <v>49</v>
+      </c>
       <c r="AL416" t="s">
-        <v>1413</v>
+        <v>1243</v>
       </c>
       <c r="AM416">
         <v>17</v>
@@ -40939,14 +40942,11 @@
       <c r="K417">
         <v>210</v>
       </c>
-      <c r="AK417">
-        <v>160</v>
-      </c>
       <c r="AL417" t="s">
-        <v>894</v>
+        <v>1413</v>
       </c>
       <c r="AM417">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="418" spans="1:39" x14ac:dyDescent="0.25">
@@ -40988,13 +40988,13 @@
         <v>1172</v>
       </c>
       <c r="AK418">
-        <v>28</v>
+        <v>160</v>
       </c>
       <c r="AL418" t="s">
-        <v>1246</v>
+        <v>894</v>
       </c>
       <c r="AM418">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="419" spans="1:39" x14ac:dyDescent="0.25">
@@ -41033,10 +41033,10 @@
         <v>300</v>
       </c>
       <c r="AK419">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="AL419" t="s">
-        <v>1275</v>
+        <v>1246</v>
       </c>
       <c r="AM419">
         <v>19</v>
@@ -41078,10 +41078,10 @@
         <v>500</v>
       </c>
       <c r="AK420">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AL420" t="s">
-        <v>1270</v>
+        <v>1275</v>
       </c>
       <c r="AM420">
         <v>19</v>
@@ -41123,10 +41123,10 @@
         <v>300</v>
       </c>
       <c r="AK421">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="AL421" t="s">
-        <v>1236</v>
+        <v>1270</v>
       </c>
       <c r="AM421">
         <v>19</v>
@@ -41171,13 +41171,13 @@
         <v>1172</v>
       </c>
       <c r="AK422">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="AL422" t="s">
-        <v>1365</v>
+        <v>1236</v>
       </c>
       <c r="AM422">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="423" spans="1:39" x14ac:dyDescent="0.25">
@@ -41225,13 +41225,13 @@
         <v>1186</v>
       </c>
       <c r="AK423">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="AL423" t="s">
-        <v>1274</v>
+        <v>1365</v>
       </c>
       <c r="AM423">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="424" spans="1:39" x14ac:dyDescent="0.25">
@@ -41279,13 +41279,13 @@
         <v>1186</v>
       </c>
       <c r="AK424">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="AL424" t="s">
-        <v>1224</v>
+        <v>1274</v>
       </c>
       <c r="AM424">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="425" spans="1:39" x14ac:dyDescent="0.25">
@@ -41336,13 +41336,13 @@
         <v>1187</v>
       </c>
       <c r="AK425">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="AL425" t="s">
-        <v>1272</v>
+        <v>1224</v>
       </c>
       <c r="AM425">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="426" spans="1:39" x14ac:dyDescent="0.25">
@@ -41389,11 +41389,14 @@
       <c r="N426" t="s">
         <v>1188</v>
       </c>
+      <c r="AK426">
+        <v>40</v>
+      </c>
       <c r="AL426" t="s">
-        <v>1369</v>
+        <v>1272</v>
       </c>
       <c r="AM426">
-        <v>47</v>
+        <v>29</v>
       </c>
     </row>
     <row r="427" spans="1:39" x14ac:dyDescent="0.25">
@@ -41439,6 +41442,12 @@
       </c>
       <c r="N427" t="s">
         <v>1188</v>
+      </c>
+      <c r="AL427" t="s">
+        <v>1369</v>
+      </c>
+      <c r="AM427">
+        <v>47</v>
       </c>
     </row>
     <row r="428" spans="1:39" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Tons of changes on E4 stuff and everything!
</commit_message>
<xml_diff>
--- a/stuff/pokemon game.xlsx
+++ b/stuff/pokemon game.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shaej\git\PokemonGame\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEDEF6F5-D581-452F-A30F-83A192452C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB24713A-C9AB-47E9-A887-A57585FA3181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7BD02A17-B686-4FC4-8065-C777F779E0C9}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{7BD02A17-B686-4FC4-8065-C777F779E0C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -6091,9 +6091,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CCD2C10-9C1D-4BA8-9034-8E41B08DF934}">
   <dimension ref="A1:AW620"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" style="1" customWidth="1"/>
     <col min="5" max="5" width="11" style="2" customWidth="1"/>
     <col min="6" max="6" width="11" style="3" customWidth="1"/>
@@ -6103,24 +6103,24 @@
     <col min="10" max="10" width="11" style="6" customWidth="1"/>
     <col min="11" max="11" width="11" customWidth="1"/>
     <col min="12" max="13" width="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.28515625" customWidth="1"/>
-    <col min="15" max="15" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.33203125" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.44140625" customWidth="1"/>
     <col min="21" max="21" width="17" customWidth="1"/>
     <col min="23" max="23" width="15" customWidth="1"/>
-    <col min="26" max="26" width="6.7109375" customWidth="1"/>
-    <col min="27" max="29" width="10.85546875" customWidth="1"/>
-    <col min="30" max="32" width="7.7109375" customWidth="1"/>
-    <col min="33" max="33" width="11.42578125" customWidth="1"/>
-    <col min="34" max="36" width="7.7109375" customWidth="1"/>
-    <col min="37" max="37" width="9.5703125" customWidth="1"/>
-    <col min="38" max="38" width="8.28515625" customWidth="1"/>
-    <col min="39" max="47" width="7.7109375" customWidth="1"/>
+    <col min="26" max="26" width="6.6640625" customWidth="1"/>
+    <col min="27" max="29" width="10.88671875" customWidth="1"/>
+    <col min="30" max="32" width="7.6640625" customWidth="1"/>
+    <col min="33" max="33" width="11.44140625" customWidth="1"/>
+    <col min="34" max="36" width="7.6640625" customWidth="1"/>
+    <col min="37" max="37" width="9.5546875" customWidth="1"/>
+    <col min="38" max="38" width="8.33203125" customWidth="1"/>
+    <col min="39" max="47" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>-1</v>
       </c>
@@ -6238,7 +6238,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="2" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B2">
         <v>-2</v>
       </c>
@@ -6309,7 +6309,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="3" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>-3</v>
       </c>
@@ -6385,7 +6385,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="4" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>-4</v>
       </c>
@@ -6456,7 +6456,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="5" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>-5</v>
       </c>
@@ -6532,7 +6532,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="6" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>-6</v>
       </c>
@@ -6602,7 +6602,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="7" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>-7</v>
       </c>
@@ -6672,7 +6672,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="8" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>-8</v>
       </c>
@@ -6746,7 +6746,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="9" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>-9</v>
       </c>
@@ -6818,7 +6818,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="10" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>-10</v>
       </c>
@@ -6885,7 +6885,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="11" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>-11</v>
       </c>
@@ -6949,7 +6949,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="12" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>-12</v>
       </c>
@@ -7012,7 +7012,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="13" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>-13</v>
       </c>
@@ -7081,7 +7081,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>-14</v>
       </c>
@@ -7141,7 +7141,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="15" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>-15</v>
       </c>
@@ -7199,7 +7199,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="16" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>-16</v>
       </c>
@@ -7254,7 +7254,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="17" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>-17</v>
       </c>
@@ -7317,7 +7317,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="18" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>-18</v>
       </c>
@@ -7386,7 +7386,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="19" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>-19</v>
       </c>
@@ -7453,7 +7453,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="20" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>-20</v>
       </c>
@@ -7517,7 +7517,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="21" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>-21</v>
       </c>
@@ -7573,7 +7573,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="22" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>-22</v>
       </c>
@@ -7622,7 +7622,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="23" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>-23</v>
       </c>
@@ -7670,7 +7670,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="24" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>-24</v>
       </c>
@@ -7718,7 +7718,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="25" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B25">
         <v>-25</v>
       </c>
@@ -7766,7 +7766,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="26" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B26">
         <v>-26</v>
       </c>
@@ -7811,7 +7811,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="27" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B27">
         <v>-27</v>
       </c>
@@ -7856,7 +7856,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="28" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>-28</v>
       </c>
@@ -7901,7 +7901,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="29" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B29">
         <v>-29</v>
       </c>
@@ -7985,7 +7985,7 @@
         <v>1494</v>
       </c>
     </row>
-    <row r="30" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>-30</v>
       </c>
@@ -8061,7 +8061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B31">
         <v>-31</v>
       </c>
@@ -8149,7 +8149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:49" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:49" x14ac:dyDescent="0.3">
       <c r="B32">
         <v>-32</v>
       </c>
@@ -8231,7 +8231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B33">
         <v>-33</v>
       </c>
@@ -8325,7 +8325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>-34</v>
       </c>
@@ -8416,7 +8416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B35">
         <v>-35</v>
       </c>
@@ -8507,7 +8507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B36">
         <v>-36</v>
       </c>
@@ -8598,7 +8598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B37">
         <v>-37</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B38">
         <v>-38</v>
       </c>
@@ -8777,7 +8777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B39">
         <v>-39</v>
       </c>
@@ -8865,7 +8865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B40">
         <v>-40</v>
       </c>
@@ -8953,7 +8953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B41">
         <v>-41</v>
       </c>
@@ -9035,7 +9035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B42">
         <v>-42</v>
       </c>
@@ -9114,7 +9114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B43">
         <v>-43</v>
       </c>
@@ -9190,7 +9190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B44">
         <v>-44</v>
       </c>
@@ -9263,7 +9263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B45">
         <v>-45</v>
       </c>
@@ -9339,7 +9339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B46">
         <v>-46</v>
       </c>
@@ -9415,7 +9415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B47">
         <v>-47</v>
       </c>
@@ -9491,7 +9491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B48">
         <v>-48</v>
       </c>
@@ -9564,7 +9564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B49">
         <v>-49</v>
       </c>
@@ -9637,7 +9637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B50">
         <v>-50</v>
       </c>
@@ -9713,7 +9713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B51">
         <v>-51</v>
       </c>
@@ -9786,7 +9786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B52">
         <v>-52</v>
       </c>
@@ -9859,7 +9859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B53">
         <v>-53</v>
       </c>
@@ -9932,7 +9932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B54">
         <v>-54</v>
       </c>
@@ -10029,7 +10029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B55">
         <v>-55</v>
       </c>
@@ -10126,7 +10126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B56">
         <v>-56</v>
       </c>
@@ -10223,7 +10223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B57">
         <v>-57</v>
       </c>
@@ -10323,7 +10323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B58">
         <v>-58</v>
       </c>
@@ -10420,7 +10420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B59">
         <v>-59</v>
       </c>
@@ -10517,7 +10517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B60">
         <v>-60</v>
       </c>
@@ -10617,7 +10617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B61">
         <v>-61</v>
       </c>
@@ -10717,7 +10717,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="62" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B62">
         <v>-62</v>
       </c>
@@ -10814,7 +10814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B63">
         <v>-63</v>
       </c>
@@ -10911,7 +10911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B64">
         <v>-64</v>
       </c>
@@ -11008,7 +11008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B65">
         <v>-65</v>
       </c>
@@ -11105,7 +11105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B66">
         <v>-66</v>
       </c>
@@ -11205,7 +11205,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="67" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B67">
         <v>-67</v>
       </c>
@@ -11305,7 +11305,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="68" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B68">
         <v>-68</v>
       </c>
@@ -11405,7 +11405,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="69" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B69">
         <v>-69</v>
       </c>
@@ -11502,7 +11502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B70">
         <v>-70</v>
       </c>
@@ -11599,7 +11599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B71">
         <v>-71</v>
       </c>
@@ -11696,7 +11696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B72">
         <v>-72</v>
       </c>
@@ -11793,7 +11793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B73">
         <v>-73</v>
       </c>
@@ -11890,7 +11890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B74">
         <v>-74</v>
       </c>
@@ -11990,7 +11990,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="75" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B75">
         <v>-75</v>
       </c>
@@ -12094,7 +12094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B76">
         <v>-76</v>
       </c>
@@ -12167,7 +12167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B77">
         <v>-77</v>
       </c>
@@ -12240,7 +12240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B78">
         <v>-78</v>
       </c>
@@ -12316,7 +12316,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="79" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B79">
         <v>-79</v>
       </c>
@@ -12389,7 +12389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B80">
         <v>-80</v>
       </c>
@@ -12462,7 +12462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B81">
         <v>-81</v>
       </c>
@@ -12535,7 +12535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B82">
         <v>-82</v>
       </c>
@@ -12608,7 +12608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B83">
         <v>-83</v>
       </c>
@@ -12681,7 +12681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B84">
         <v>-84</v>
       </c>
@@ -12757,7 +12757,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="85" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B85">
         <v>-85</v>
       </c>
@@ -12833,7 +12833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B86">
         <v>-86</v>
       </c>
@@ -12909,7 +12909,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="87" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B87">
         <v>-87</v>
       </c>
@@ -12982,7 +12982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B88">
         <v>-88</v>
       </c>
@@ -13055,7 +13055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B89">
         <v>-89</v>
       </c>
@@ -13131,7 +13131,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="90" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B90">
         <v>-90</v>
       </c>
@@ -13207,7 +13207,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="91" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B91">
         <v>-91</v>
       </c>
@@ -13283,7 +13283,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="92" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B92">
         <v>-92</v>
       </c>
@@ -13356,7 +13356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B93">
         <v>-93</v>
       </c>
@@ -13429,7 +13429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B94">
         <v>-94</v>
       </c>
@@ -13502,7 +13502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B95">
         <v>-95</v>
       </c>
@@ -13575,7 +13575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B96">
         <v>-96</v>
       </c>
@@ -13648,7 +13648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B97">
         <v>-97</v>
       </c>
@@ -13721,7 +13721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B98">
         <v>-98</v>
       </c>
@@ -13794,7 +13794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B99">
         <v>-99</v>
       </c>
@@ -13867,7 +13867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B100">
         <v>-100</v>
       </c>
@@ -13943,7 +13943,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="101" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B101">
         <v>-101</v>
       </c>
@@ -14019,7 +14019,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="102" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B102">
         <v>-102</v>
       </c>
@@ -14095,7 +14095,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="103" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B103">
         <v>-103</v>
       </c>
@@ -14174,7 +14174,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="104" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B104">
         <v>-104</v>
       </c>
@@ -14250,7 +14250,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="105" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B105">
         <v>-105</v>
       </c>
@@ -14323,7 +14323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B106">
         <v>-106</v>
       </c>
@@ -14396,7 +14396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B107">
         <v>-107</v>
       </c>
@@ -14469,7 +14469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B108">
         <v>-108</v>
       </c>
@@ -14542,7 +14542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B109">
         <v>-109</v>
       </c>
@@ -14615,7 +14615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B110">
         <v>-110</v>
       </c>
@@ -14691,7 +14691,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="111" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B111">
         <v>-111</v>
       </c>
@@ -14764,7 +14764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B112">
         <v>-112</v>
       </c>
@@ -14840,7 +14840,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="113" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B113">
         <v>-113</v>
       </c>
@@ -14916,7 +14916,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="114" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B114">
         <v>-114</v>
       </c>
@@ -14989,7 +14989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B115">
         <v>-115</v>
       </c>
@@ -15062,7 +15062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B116">
         <v>-116</v>
       </c>
@@ -15135,7 +15135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B117">
         <v>-117</v>
       </c>
@@ -15208,7 +15208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B118">
         <v>-118</v>
       </c>
@@ -15281,7 +15281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B119">
         <v>-119</v>
       </c>
@@ -15354,7 +15354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B120">
         <v>-120</v>
       </c>
@@ -15427,7 +15427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B121">
         <v>-121</v>
       </c>
@@ -15500,7 +15500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B122">
         <v>-122</v>
       </c>
@@ -15573,7 +15573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B123">
         <v>-123</v>
       </c>
@@ -15646,7 +15646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B124">
         <v>-124</v>
       </c>
@@ -15719,7 +15719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B125">
         <v>-125</v>
       </c>
@@ -15795,7 +15795,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="126" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B126">
         <v>-126</v>
       </c>
@@ -15868,7 +15868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B127">
         <v>-127</v>
       </c>
@@ -15941,7 +15941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="2:40" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:40" x14ac:dyDescent="0.3">
       <c r="B128">
         <v>-128</v>
       </c>
@@ -16014,7 +16014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B129">
         <v>-129</v>
       </c>
@@ -16087,7 +16087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B130">
         <v>-130</v>
       </c>
@@ -16160,7 +16160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B131">
         <v>-131</v>
       </c>
@@ -16233,7 +16233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B132">
         <v>-132</v>
       </c>
@@ -16306,7 +16306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B133">
         <v>-133</v>
       </c>
@@ -16379,7 +16379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B134">
         <v>-134</v>
       </c>
@@ -16452,7 +16452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B135">
         <v>-135</v>
       </c>
@@ -16525,7 +16525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B136">
         <v>-136</v>
       </c>
@@ -16598,7 +16598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B137">
         <v>-137</v>
       </c>
@@ -16671,7 +16671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B138">
         <v>-138</v>
       </c>
@@ -16744,7 +16744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B139">
         <v>-139</v>
       </c>
@@ -16814,7 +16814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B140">
         <v>-140</v>
       </c>
@@ -16884,7 +16884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B141">
         <v>-141</v>
       </c>
@@ -16961,7 +16961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B142">
         <v>-142</v>
       </c>
@@ -17041,7 +17041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B143">
         <v>-143</v>
       </c>
@@ -17121,7 +17121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:39" x14ac:dyDescent="0.3">
       <c r="B144">
         <v>-144</v>
       </c>
@@ -17213,7 +17213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>1190</v>
       </c>
@@ -17298,7 +17298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>1</v>
       </c>
@@ -17408,7 +17408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>2</v>
       </c>
@@ -17515,7 +17515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>3</v>
       </c>
@@ -17622,7 +17622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>4</v>
       </c>
@@ -17729,7 +17729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>5</v>
       </c>
@@ -17836,7 +17836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>6</v>
       </c>
@@ -17940,7 +17940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>7</v>
       </c>
@@ -18053,7 +18053,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="153" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>8</v>
       </c>
@@ -18163,7 +18163,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="154" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>9</v>
       </c>
@@ -18267,7 +18267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>13</v>
       </c>
@@ -18374,7 +18374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>14</v>
       </c>
@@ -18481,7 +18481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>15</v>
       </c>
@@ -18588,7 +18588,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>10</v>
       </c>
@@ -18695,7 +18695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>11</v>
       </c>
@@ -18802,7 +18802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>12</v>
       </c>
@@ -18906,7 +18906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>16</v>
       </c>
@@ -19013,7 +19013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>17</v>
       </c>
@@ -19120,7 +19120,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>18</v>
       </c>
@@ -19230,7 +19230,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="164" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>41</v>
       </c>
@@ -19340,7 +19340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>42</v>
       </c>
@@ -19447,7 +19447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>43</v>
       </c>
@@ -19551,7 +19551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>19</v>
       </c>
@@ -19656,7 +19656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>20</v>
       </c>
@@ -19764,7 +19764,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="169" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>21</v>
       </c>
@@ -19871,7 +19871,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="170" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>22</v>
       </c>
@@ -19978,7 +19978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>26</v>
       </c>
@@ -20083,7 +20083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>27</v>
       </c>
@@ -20188,7 +20188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>28</v>
       </c>
@@ -20287,7 +20287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>29</v>
       </c>
@@ -20391,7 +20391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>30</v>
       </c>
@@ -20495,7 +20495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>31</v>
       </c>
@@ -20596,7 +20596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>32</v>
       </c>
@@ -20698,7 +20698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>33</v>
       </c>
@@ -20800,7 +20800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>34</v>
       </c>
@@ -20899,7 +20899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>122</v>
       </c>
@@ -21001,7 +21001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>123</v>
       </c>
@@ -21103,7 +21103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>124</v>
       </c>
@@ -21202,7 +21202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>38</v>
       </c>
@@ -21303,7 +21303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>39</v>
       </c>
@@ -21410,7 +21410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>40</v>
       </c>
@@ -21517,7 +21517,7 @@
         <v>1557</v>
       </c>
     </row>
-    <row r="186" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>35</v>
       </c>
@@ -21621,7 +21621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>36</v>
       </c>
@@ -21725,7 +21725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>37</v>
       </c>
@@ -21826,7 +21826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>60</v>
       </c>
@@ -21928,7 +21928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>61</v>
       </c>
@@ -22030,7 +22030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>62</v>
       </c>
@@ -22129,7 +22129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>129</v>
       </c>
@@ -22227,7 +22227,7 @@
         <v>1557</v>
       </c>
     </row>
-    <row r="193" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>125</v>
       </c>
@@ -22328,7 +22328,7 @@
         <v>1557</v>
       </c>
     </row>
-    <row r="194" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>126</v>
       </c>
@@ -22432,7 +22432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>127</v>
       </c>
@@ -22533,7 +22533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>128</v>
       </c>
@@ -22637,7 +22637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>107</v>
       </c>
@@ -22741,7 +22741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>108</v>
       </c>
@@ -22845,7 +22845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>109</v>
       </c>
@@ -22946,7 +22946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>130</v>
       </c>
@@ -23053,7 +23053,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="201" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>131</v>
       </c>
@@ -23154,7 +23154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>180</v>
       </c>
@@ -23255,7 +23255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>181</v>
       </c>
@@ -23353,7 +23353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>84</v>
       </c>
@@ -23454,7 +23454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>85</v>
       </c>
@@ -23552,7 +23552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>204</v>
       </c>
@@ -23650,7 +23650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>162</v>
       </c>
@@ -23751,7 +23751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>163</v>
       </c>
@@ -23846,7 +23846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>205</v>
       </c>
@@ -23942,7 +23942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>206</v>
       </c>
@@ -24035,7 +24035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>207</v>
       </c>
@@ -24133,7 +24133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>208</v>
       </c>
@@ -24228,7 +24228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>186</v>
       </c>
@@ -24329,7 +24329,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="214" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>187</v>
       </c>
@@ -24427,7 +24427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>188</v>
       </c>
@@ -24522,7 +24522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>81</v>
       </c>
@@ -24620,7 +24620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="217" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>82</v>
       </c>
@@ -24718,7 +24718,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="218" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>94</v>
       </c>
@@ -24822,7 +24822,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="219" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>95</v>
       </c>
@@ -24923,7 +24923,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="220" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>49</v>
       </c>
@@ -25021,7 +25021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>50</v>
       </c>
@@ -25122,7 +25122,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="222" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>51</v>
       </c>
@@ -25217,7 +25217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>189</v>
       </c>
@@ -25321,7 +25321,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="224" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>190</v>
       </c>
@@ -25419,7 +25419,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="225" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>178</v>
       </c>
@@ -25520,7 +25520,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="226" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>179</v>
       </c>
@@ -25615,7 +25615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="227" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>132</v>
       </c>
@@ -25710,7 +25710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>133</v>
       </c>
@@ -25808,7 +25808,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>134</v>
       </c>
@@ -25918,7 +25918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>63</v>
       </c>
@@ -26025,7 +26025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>64</v>
       </c>
@@ -26132,7 +26132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>65</v>
       </c>
@@ -26236,7 +26236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>66</v>
       </c>
@@ -26343,7 +26343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>83</v>
       </c>
@@ -26450,7 +26450,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="235" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>137</v>
       </c>
@@ -26560,7 +26560,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="236" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>138</v>
       </c>
@@ -26664,7 +26664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>52</v>
       </c>
@@ -26774,7 +26774,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="238" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>53</v>
       </c>
@@ -26881,7 +26881,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="239" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>54</v>
       </c>
@@ -26991,7 +26991,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="240" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>55</v>
       </c>
@@ -27101,7 +27101,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="241" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>56</v>
       </c>
@@ -27208,7 +27208,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="242" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>191</v>
       </c>
@@ -27309,7 +27309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>209</v>
       </c>
@@ -27412,7 +27412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>210</v>
       </c>
@@ -27517,7 +27517,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="245" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>211</v>
       </c>
@@ -27616,7 +27616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>101</v>
       </c>
@@ -27720,7 +27720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>102</v>
       </c>
@@ -27827,7 +27827,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="248" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>103</v>
       </c>
@@ -27931,7 +27931,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="249" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>96</v>
       </c>
@@ -28041,7 +28041,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="250" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>97</v>
       </c>
@@ -28148,7 +28148,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="251" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>92</v>
       </c>
@@ -28252,7 +28252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>93</v>
       </c>
@@ -28356,7 +28356,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="253" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>110</v>
       </c>
@@ -28449,7 +28449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>111</v>
       </c>
@@ -28551,7 +28551,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="255" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>112</v>
       </c>
@@ -28656,7 +28656,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="256" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>164</v>
       </c>
@@ -28763,7 +28763,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="257" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>165</v>
       </c>
@@ -28867,7 +28867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="258" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>166</v>
       </c>
@@ -28968,7 +28968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>139</v>
       </c>
@@ -29072,7 +29072,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="260" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>140</v>
       </c>
@@ -29176,7 +29176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>141</v>
       </c>
@@ -29277,7 +29277,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="262" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>151</v>
       </c>
@@ -29384,7 +29384,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="263" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>152</v>
       </c>
@@ -29491,7 +29491,7 @@
         <v>1558</v>
       </c>
     </row>
-    <row r="264" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>153</v>
       </c>
@@ -29598,7 +29598,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="265" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>142</v>
       </c>
@@ -29706,7 +29706,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="266" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>143</v>
       </c>
@@ -29814,7 +29814,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="267" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>144</v>
       </c>
@@ -29916,7 +29916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>145</v>
       </c>
@@ -30021,7 +30021,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="269" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>146</v>
       </c>
@@ -30123,7 +30123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="270" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>147</v>
       </c>
@@ -30225,7 +30225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>148</v>
       </c>
@@ -30330,7 +30330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="272" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>149</v>
       </c>
@@ -30423,7 +30423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="273" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>150</v>
       </c>
@@ -30513,7 +30513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="274" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>78</v>
       </c>
@@ -30606,7 +30606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>79</v>
       </c>
@@ -30696,7 +30696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>80</v>
       </c>
@@ -30795,7 +30795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="277" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>192</v>
       </c>
@@ -30897,7 +30897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>193</v>
       </c>
@@ -30996,7 +30996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>154</v>
       </c>
@@ -31098,7 +31098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="280" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>155</v>
       </c>
@@ -31197,7 +31197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="281" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>156</v>
       </c>
@@ -31296,7 +31296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="282" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>167</v>
       </c>
@@ -31398,7 +31398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>168</v>
       </c>
@@ -31497,7 +31497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="284" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>182</v>
       </c>
@@ -31598,7 +31598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>183</v>
       </c>
@@ -31696,7 +31696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>212</v>
       </c>
@@ -31795,7 +31795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>213</v>
       </c>
@@ -31891,7 +31891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>159</v>
       </c>
@@ -31990,7 +31990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="289" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>160</v>
       </c>
@@ -32089,7 +32089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="290" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>161</v>
       </c>
@@ -32185,7 +32185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="291" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>174</v>
       </c>
@@ -32284,7 +32284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="292" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>175</v>
       </c>
@@ -32380,7 +32380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="293" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>176</v>
       </c>
@@ -32479,7 +32479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>177</v>
       </c>
@@ -32575,7 +32575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>217</v>
       </c>
@@ -32671,7 +32671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="296" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>44</v>
       </c>
@@ -32775,7 +32775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>45</v>
       </c>
@@ -32876,7 +32876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>119</v>
       </c>
@@ -32980,7 +32980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="299" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>120</v>
       </c>
@@ -33084,7 +33084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>121</v>
       </c>
@@ -33185,7 +33185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>194</v>
       </c>
@@ -33289,7 +33289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>195</v>
       </c>
@@ -33390,7 +33390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>196</v>
       </c>
@@ -33497,7 +33497,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="304" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>197</v>
       </c>
@@ -33601,7 +33601,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="305" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>169</v>
       </c>
@@ -33703,7 +33703,7 @@
         <v>1562</v>
       </c>
     </row>
-    <row r="306" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>170</v>
       </c>
@@ -33805,7 +33805,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="307" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>171</v>
       </c>
@@ -33907,7 +33907,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="308" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>72</v>
       </c>
@@ -34009,7 +34009,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="309" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>73</v>
       </c>
@@ -34111,7 +34111,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="310" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>74</v>
       </c>
@@ -34210,7 +34210,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="311" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>75</v>
       </c>
@@ -34314,7 +34314,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="312" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>76</v>
       </c>
@@ -34418,7 +34418,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="313" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>77</v>
       </c>
@@ -34516,7 +34516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="314" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>115</v>
       </c>
@@ -34617,7 +34617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>116</v>
       </c>
@@ -34715,7 +34715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>69</v>
       </c>
@@ -34816,7 +34816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="317" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>70</v>
       </c>
@@ -34917,7 +34917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>71</v>
       </c>
@@ -35015,7 +35015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="319" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>57</v>
       </c>
@@ -35114,7 +35114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>58</v>
       </c>
@@ -35213,7 +35213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>59</v>
       </c>
@@ -35309,7 +35309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="322" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>67</v>
       </c>
@@ -35408,7 +35408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="323" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>68</v>
       </c>
@@ -35504,7 +35504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="324" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>117</v>
       </c>
@@ -35603,7 +35603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="325" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>118</v>
       </c>
@@ -35699,7 +35699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="326" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>214</v>
       </c>
@@ -35769,7 +35769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="327" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>215</v>
       </c>
@@ -35842,7 +35842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="328" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>216</v>
       </c>
@@ -35915,7 +35915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="329" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>228</v>
       </c>
@@ -35980,7 +35980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>229</v>
       </c>
@@ -36045,7 +36045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="331" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>230</v>
       </c>
@@ -36110,7 +36110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="332" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>231</v>
       </c>
@@ -36178,7 +36178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="333" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>232</v>
       </c>
@@ -36246,7 +36246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="334" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>233</v>
       </c>
@@ -36311,7 +36311,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="335" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>225</v>
       </c>
@@ -36375,7 +36375,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="336" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>226</v>
       </c>
@@ -36445,7 +36445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="337" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>227</v>
       </c>
@@ -36515,7 +36515,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="338" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>218</v>
       </c>
@@ -36588,7 +36588,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="339" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>219</v>
       </c>
@@ -36661,7 +36661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="340" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>223</v>
       </c>
@@ -36743,7 +36743,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="341" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>224</v>
       </c>
@@ -36819,7 +36819,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="342" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A342" s="10">
         <v>-10</v>
       </c>
@@ -36889,7 +36889,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="343" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A343" s="10">
         <v>-11</v>
       </c>
@@ -36971,7 +36971,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="344" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A344" s="10">
         <v>-7</v>
       </c>
@@ -37041,7 +37041,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="345" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A345" s="10">
         <v>-8</v>
       </c>
@@ -37109,7 +37109,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="346" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A346" s="10">
         <v>-9</v>
       </c>
@@ -37170,7 +37170,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="347" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A347" s="10">
         <v>-14</v>
       </c>
@@ -37232,7 +37232,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="348" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A348" s="10">
         <v>-15</v>
       </c>
@@ -37294,7 +37294,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="349" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A349" s="10">
         <v>-16</v>
       </c>
@@ -37353,7 +37353,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="350" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A350" s="10">
         <v>-1</v>
       </c>
@@ -37415,7 +37415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="351" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A351" s="10">
         <v>-2</v>
       </c>
@@ -37477,7 +37477,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="352" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A352" s="10">
         <v>-3</v>
       </c>
@@ -37536,7 +37536,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="353" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A353" s="10">
         <v>-4</v>
       </c>
@@ -37598,7 +37598,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="354" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A354" s="10">
         <v>-5</v>
       </c>
@@ -37660,7 +37660,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="355" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A355" s="10">
         <v>-6</v>
       </c>
@@ -37722,7 +37722,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="356" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A356" s="10">
         <v>-17</v>
       </c>
@@ -37783,7 +37783,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="357" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A357" s="10">
         <v>-18</v>
       </c>
@@ -37847,7 +37847,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="358" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A358" s="48">
         <v>-17</v>
       </c>
@@ -37908,7 +37908,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="359" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A359" s="48">
         <v>-18</v>
       </c>
@@ -37972,7 +37972,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="360" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A360" s="48">
         <v>-15</v>
       </c>
@@ -38031,7 +38031,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="361" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A361" s="48">
         <v>-16</v>
       </c>
@@ -38093,7 +38093,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="362" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A362" s="48">
         <v>-1</v>
       </c>
@@ -38151,7 +38151,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="363" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A363" s="48">
         <v>-2</v>
       </c>
@@ -38212,7 +38212,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="364" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A364" s="48">
         <v>-3</v>
       </c>
@@ -38273,7 +38273,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="365" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A365" s="48">
         <v>-12</v>
       </c>
@@ -38331,7 +38331,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="366" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A366" s="48">
         <v>-13</v>
       </c>
@@ -38389,7 +38389,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="367" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A367" s="48">
         <v>-14</v>
       </c>
@@ -38450,7 +38450,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="368" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A368" s="48">
         <v>-4</v>
       </c>
@@ -38514,7 +38514,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="369" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A369" s="48">
         <v>-5</v>
       </c>
@@ -38578,7 +38578,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="370" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A370" s="48">
         <v>-6</v>
       </c>
@@ -38639,7 +38639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="371" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A371" s="48">
         <v>-7</v>
       </c>
@@ -38703,7 +38703,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="372" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A372" s="48">
         <v>-8</v>
       </c>
@@ -38764,7 +38764,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="373" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A373">
         <v>243</v>
       </c>
@@ -38823,7 +38823,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="374" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A374">
         <v>240</v>
       </c>
@@ -38882,7 +38882,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="375" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A375">
         <v>244</v>
       </c>
@@ -38941,7 +38941,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="376" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A376">
         <v>242</v>
       </c>
@@ -38997,7 +38997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="377" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A377">
         <v>241</v>
       </c>
@@ -39056,7 +39056,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="378" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A378">
         <v>245</v>
       </c>
@@ -39115,7 +39115,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="379" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A379">
         <v>246</v>
       </c>
@@ -39174,7 +39174,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="380" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A380">
         <v>247</v>
       </c>
@@ -39233,7 +39233,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="381" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A381">
         <v>249</v>
       </c>
@@ -39292,7 +39292,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="382" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:40" x14ac:dyDescent="0.3">
       <c r="B382">
         <v>237</v>
       </c>
@@ -39344,7 +39344,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="383" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A383">
         <v>89</v>
       </c>
@@ -39398,7 +39398,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="384" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A384">
         <v>90</v>
       </c>
@@ -39455,7 +39455,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="385" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A385">
         <v>91</v>
       </c>
@@ -39512,7 +39512,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="386" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A386">
         <v>198</v>
       </c>
@@ -39560,7 +39560,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="387" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A387">
         <v>199</v>
       </c>
@@ -39608,7 +39608,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="388" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A388">
         <v>46</v>
       </c>
@@ -39653,7 +39653,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="389" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A389">
         <v>47</v>
       </c>
@@ -39698,7 +39698,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="390" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A390">
         <v>48</v>
       </c>
@@ -39743,7 +39743,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="391" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A391">
         <v>220</v>
       </c>
@@ -39788,7 +39788,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="392" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A392">
         <v>200</v>
       </c>
@@ -39833,7 +39833,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="393" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A393">
         <v>201</v>
       </c>
@@ -39878,7 +39878,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="394" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A394">
         <v>202</v>
       </c>
@@ -39923,7 +39923,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="395" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A395">
         <v>203</v>
       </c>
@@ -39968,7 +39968,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="396" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A396" s="49">
         <v>-3</v>
       </c>
@@ -40013,7 +40013,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="397" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A397" s="49">
         <v>-4</v>
       </c>
@@ -40061,7 +40061,7 @@
         <v>1556</v>
       </c>
     </row>
-    <row r="398" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A398" s="49">
         <v>-5</v>
       </c>
@@ -40106,7 +40106,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="399" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A399">
         <v>86</v>
       </c>
@@ -40151,7 +40151,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="400" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A400">
         <v>87</v>
       </c>
@@ -40196,7 +40196,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="401" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A401">
         <v>88</v>
       </c>
@@ -40241,7 +40241,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="402" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A402">
         <v>172</v>
       </c>
@@ -40286,7 +40286,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="403" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A403">
         <v>173</v>
       </c>
@@ -40331,7 +40331,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="404" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A404" s="49">
         <v>-6</v>
       </c>
@@ -40376,7 +40376,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="405" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A405" s="49">
         <v>-7</v>
       </c>
@@ -40421,7 +40421,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="406" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A406">
         <v>157</v>
       </c>
@@ -40466,7 +40466,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="407" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A407">
         <v>158</v>
       </c>
@@ -40511,7 +40511,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="408" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A408">
         <v>221</v>
       </c>
@@ -40556,7 +40556,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="409" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A409">
         <v>222</v>
       </c>
@@ -40601,7 +40601,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="410" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A410">
         <v>184</v>
       </c>
@@ -40652,7 +40652,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="411" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A411">
         <v>185</v>
       </c>
@@ -40700,7 +40700,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="412" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A412" s="10">
         <v>-12</v>
       </c>
@@ -40745,7 +40745,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="413" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A413" s="10">
         <v>-13</v>
       </c>
@@ -40790,7 +40790,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="414" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A414">
         <v>23</v>
       </c>
@@ -40832,7 +40832,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="415" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A415" s="49">
         <v>-1</v>
       </c>
@@ -40874,7 +40874,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="416" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A416" s="49">
         <v>-2</v>
       </c>
@@ -40919,7 +40919,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="417" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A417">
         <v>24</v>
       </c>
@@ -40964,7 +40964,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="418" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A418">
         <v>25</v>
       </c>
@@ -41009,7 +41009,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="419" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A419" s="49">
         <v>-8</v>
       </c>
@@ -41054,7 +41054,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="420" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A420" s="49">
         <v>-9</v>
       </c>
@@ -41099,7 +41099,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="421" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A421">
         <v>113</v>
       </c>
@@ -41144,7 +41144,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="422" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A422">
         <v>114</v>
       </c>
@@ -41192,7 +41192,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="423" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A423">
         <v>98</v>
       </c>
@@ -41246,7 +41246,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="424" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A424">
         <v>99</v>
       </c>
@@ -41300,7 +41300,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="425" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A425">
         <v>100</v>
       </c>
@@ -41357,7 +41357,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="426" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A426" s="48">
         <v>-9</v>
       </c>
@@ -41411,7 +41411,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="427" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A427" s="48">
         <v>-10</v>
       </c>
@@ -41465,7 +41465,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="428" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A428" s="48">
         <v>-11</v>
       </c>
@@ -41519,7 +41519,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="429" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A429">
         <v>234</v>
       </c>
@@ -41555,7 +41555,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="430" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A430">
         <v>235</v>
       </c>
@@ -41591,7 +41591,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="431" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A431">
         <v>236</v>
       </c>
@@ -41627,7 +41627,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="432" spans="1:39" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A432">
         <v>237</v>
       </c>
@@ -41663,7 +41663,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="433" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A433">
         <v>238</v>
       </c>
@@ -41699,7 +41699,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="434" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A434">
         <v>239</v>
       </c>
@@ -41735,7 +41735,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="435" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A435">
         <v>248</v>
       </c>
@@ -41747,7 +41747,7 @@
       </c>
       <c r="D435" s="1">
         <f t="shared" si="21"/>
-        <v>680</v>
+        <v>640</v>
       </c>
       <c r="E435" s="2">
         <v>97</v>
@@ -41756,22 +41756,22 @@
         <v>107</v>
       </c>
       <c r="G435" s="4">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="H435" s="5">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="I435" s="4">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="J435" s="6">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="K435">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="436" spans="1:14" x14ac:dyDescent="0.25">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="436" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B436">
         <v>291</v>
       </c>
@@ -41804,7 +41804,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="437" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A437">
         <v>104</v>
       </c>
@@ -41849,7 +41849,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="438" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A438">
         <v>105</v>
       </c>
@@ -41894,7 +41894,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="439" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A439">
         <v>106</v>
       </c>
@@ -41939,7 +41939,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="440" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A440">
         <v>135</v>
       </c>
@@ -41984,7 +41984,7 @@
         <v>1122</v>
       </c>
     </row>
-    <row r="441" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A441">
         <v>136</v>
       </c>
@@ -42029,7 +42029,7 @@
         <v>1122</v>
       </c>
     </row>
-    <row r="620" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="620" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C620">
         <f>MAX(C385:C618)</f>
         <v>0</v>

</xml_diff>

<commit_message>
Sprite update and slight bug fixes
</commit_message>
<xml_diff>
--- a/stuff/pokemon game.xlsx
+++ b/stuff/pokemon game.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D3650C1-C191-48A9-8853-D4916E6771D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{571D88D8-6BFA-4649-A5DD-C9712E99DB3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7BD02A17-B686-4FC4-8065-C777F779E0C9}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3214" uniqueCount="1672">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3215" uniqueCount="1673">
   <si>
     <t>Leafer</t>
   </si>
@@ -5053,6 +5052,9 @@
   </si>
   <si>
     <t>St. Joseph 2A</t>
+  </si>
+  <si>
+    <t>St. Joseph 4A</t>
   </si>
 </sst>
 </file>
@@ -37035,6 +37037,9 @@
       <c r="U344">
         <v>1</v>
       </c>
+      <c r="V344" s="10" t="s">
+        <v>1672</v>
+      </c>
       <c r="AK344">
         <v>58</v>
       </c>

</xml_diff>